<commit_message>
Add ESTADISTICA_2026_DROPDOWN_BELLO - professional Excel with dynamic dropdown
</commit_message>
<xml_diff>
--- a/workspaces/cobranza/estadisticas/ESTADISTICA_2026_DROPDOWN_BELLO.xlsx
+++ b/workspaces/cobranza/estadisticas/ESTADISTICA_2026_DROPDOWN_BELLO.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="78">
+  <fonts count="101">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -470,8 +470,145 @@
       <color rgb="00808080"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002E5FA3"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002E5FA3"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008B0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008B0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FF8C00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="003576B6"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="003576B6"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005D3EAD"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005D3EAD"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00808080"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C9A227"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C9A227"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFD966"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002E5FA3"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008B0000"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="23">
+  <fills count="30">
     <fill>
       <patternFill/>
     </fill>
@@ -583,8 +720,43 @@
         <fgColor rgb="00F2D0D0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008B0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FADADD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003576B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005D3EAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D8E8F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0E0E0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="58">
+  <borders count="60">
     <border>
       <left/>
       <right/>
@@ -1248,11 +1420,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00666666"/>
+      </left>
+      <right style="medium">
+        <color rgb="00666666"/>
+      </right>
+      <top style="medium">
+        <color rgb="00666666"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00666666"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="287">
+  <cellXfs count="403">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -2052,6 +2252,302 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="94" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="95" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="96" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="9" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="97" fillId="15" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="98" fillId="12" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="99" fillId="22" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="47" fillId="15" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="47" fillId="19" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="47" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="47" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="11" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="56" fillId="15" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="45" fillId="14" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="46" fillId="29" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="47" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="47" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="47" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="79" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="79" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="79" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="100" fillId="9" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="8" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="83" fillId="8" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="52" fillId="8" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="85" fillId="8" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="86" fillId="8" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="87" fillId="8" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="23" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="83" fillId="23" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="52" fillId="23" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="85" fillId="23" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="86" fillId="23" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="87" fillId="23" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="78" fillId="10" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="58" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="79" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="60" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="80" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="51" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="60" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="84" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="85" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="60" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="86" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="86" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="18" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="60" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="22" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="87" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="87" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="88" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="89" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="89" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="27" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="60" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="90" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="91" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="91" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="20" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="60" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="92" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="93" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="93" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="51" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="83" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="23" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2422,38 +2918,38 @@
   <dimension ref="A1:O43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="86" t="inlineStr">
+      <c r="A1" s="287" t="inlineStr">
         <is>
           <t>PROTEG-RT MUTUALIDAD</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="87" t="inlineStr">
+      <c r="A2" s="288" t="inlineStr">
         <is>
           <t>DASHBOARD — REPORTE DE COBRANZA JUNTA MENSUAL</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="204" t="inlineStr">
+      <c r="A3" s="289" t="inlineStr">
         <is>
           <t>AÑO 2026</t>
         </is>
@@ -2476,23 +2972,23 @@
       <c r="N4" s="89" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="90" t="inlineStr">
+      <c r="A5" s="290" t="inlineStr">
         <is>
           <t>MES:</t>
         </is>
       </c>
-      <c r="C5" s="91" t="inlineStr">
+      <c r="C5" s="291" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
       <c r="D5" s="162" t="n"/>
-      <c r="E5" s="90" t="inlineStr">
+      <c r="E5" s="290" t="inlineStr">
         <is>
           <t>AÑO:</t>
         </is>
       </c>
-      <c r="G5" s="264" t="inlineStr">
+      <c r="G5" s="292" t="inlineStr">
         <is>
           <t>← Cambia el mes</t>
         </is>
@@ -2500,7 +2996,7 @@
       <c r="H5" s="162" t="n"/>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="265" t="inlineStr">
+      <c r="A7" s="293" t="inlineStr">
         <is>
           <t>COBRANZA
 TOTAL GENERAL</t>
@@ -2508,7 +3004,7 @@
       </c>
       <c r="B7" s="45" t="n"/>
       <c r="C7" s="46" t="n"/>
-      <c r="D7" s="266" t="inlineStr">
+      <c r="D7" s="293" t="inlineStr">
         <is>
           <t>COBRANZA
 RECUPERADA</t>
@@ -2516,7 +3012,7 @@
       </c>
       <c r="E7" s="45" t="n"/>
       <c r="F7" s="46" t="n"/>
-      <c r="G7" s="266" t="inlineStr">
+      <c r="G7" s="293" t="inlineStr">
         <is>
           <t>COBRANZA
 EFECTIVA</t>
@@ -2524,7 +3020,7 @@
       </c>
       <c r="H7" s="45" t="n"/>
       <c r="I7" s="46" t="n"/>
-      <c r="J7" s="266" t="inlineStr">
+      <c r="J7" s="293" t="inlineStr">
         <is>
           <t>CANCELACIONES</t>
         </is>
@@ -2535,25 +3031,25 @@
       <c r="N7" s="38" t="n"/>
     </row>
     <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="267">
+      <c r="A8" s="294">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),58,132,206,280,354,428,502,576,650,724,798,872)),"")</f>
         <v/>
       </c>
       <c r="B8" s="163" t="n"/>
       <c r="C8" s="164" t="n"/>
-      <c r="D8" s="268">
+      <c r="D8" s="294">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),49,123,197,271,345,419,493,567,641,715,789,863)),"")</f>
         <v/>
       </c>
       <c r="E8" s="171" t="n"/>
       <c r="F8" s="172" t="n"/>
-      <c r="G8" s="269">
+      <c r="G8" s="295">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),40,114,188,262,336,410,484,558,632,706,780,854)),"")</f>
         <v/>
       </c>
       <c r="H8" s="169" t="n"/>
       <c r="I8" s="170" t="n"/>
-      <c r="J8" s="270">
+      <c r="J8" s="296">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),17,96,170,244,318,392,466,540,614,688,762,836)),"")</f>
         <v/>
       </c>
@@ -2563,25 +3059,25 @@
       <c r="N8" s="38" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="271">
+      <c r="A9" s="297">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),58,132,206,280,354,428,502,576,650,724,798,872))/INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),58,132,206,280,354,428,502,576,650,724,798,872)),"")</f>
         <v/>
       </c>
       <c r="B9" s="45" t="n"/>
       <c r="C9" s="46" t="n"/>
-      <c r="D9" s="272">
+      <c r="D9" s="298">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),49,123,197,271,345,419,493,567,641,715,789,863))/INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),58,132,206,280,354,428,502,576,650,724,798,872)),"")</f>
         <v/>
       </c>
       <c r="E9" s="45" t="n"/>
       <c r="F9" s="46" t="n"/>
-      <c r="G9" s="273">
+      <c r="G9" s="299">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),40,114,188,262,336,410,484,558,632,706,780,854))/INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),58,132,206,280,354,428,502,576,650,724,798,872)),"")</f>
         <v/>
       </c>
       <c r="H9" s="45" t="n"/>
       <c r="I9" s="46" t="n"/>
-      <c r="J9" s="274">
+      <c r="J9" s="300">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),17,96,170,244,318,392,466,540,614,688,762,836))/INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),58,132,206,280,354,428,502,576,650,724,798,872)),"")</f>
         <v/>
       </c>
@@ -2607,7 +3103,7 @@
       <c r="N10" s="38" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="265" t="inlineStr">
+      <c r="A11" s="301" t="inlineStr">
         <is>
           <t>COBRANZA
 CORRIENTE</t>
@@ -2615,7 +3111,7 @@
       </c>
       <c r="B11" s="45" t="n"/>
       <c r="C11" s="46" t="n"/>
-      <c r="D11" s="266" t="inlineStr">
+      <c r="D11" s="301" t="inlineStr">
         <is>
           <t>COBRANZA
 VENCIDA</t>
@@ -2623,7 +3119,7 @@
       </c>
       <c r="E11" s="45" t="n"/>
       <c r="F11" s="46" t="n"/>
-      <c r="G11" s="266" t="inlineStr">
+      <c r="G11" s="301" t="inlineStr">
         <is>
           <t>COBRANZA
 ANTICIPADA</t>
@@ -2631,7 +3127,7 @@
       </c>
       <c r="H11" s="45" t="n"/>
       <c r="I11" s="46" t="n"/>
-      <c r="J11" s="266" t="inlineStr">
+      <c r="J11" s="301" t="inlineStr">
         <is>
           <t>PROYECCION
 SIG. MES</t>
@@ -2643,25 +3139,25 @@
       <c r="N11" s="38" t="n"/>
     </row>
     <row r="12" ht="38" customHeight="1">
-      <c r="A12" s="267">
+      <c r="A12" s="302">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),11,87,161,235,309,383,457,531,605,679,753,827)),"")</f>
         <v/>
       </c>
       <c r="B12" s="163" t="n"/>
       <c r="C12" s="164" t="n"/>
-      <c r="D12" s="275">
+      <c r="D12" s="303">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),31,105,179,253,327,401,475,549,623,697,771,845)),"")</f>
         <v/>
       </c>
       <c r="E12" s="167" t="n"/>
       <c r="F12" s="168" t="n"/>
-      <c r="G12" s="276">
+      <c r="G12" s="304">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),1,141,215,289,363,437,511,585,659,733,807,881)),"")</f>
         <v/>
       </c>
       <c r="H12" s="173" t="n"/>
       <c r="I12" s="174" t="n"/>
-      <c r="J12" s="277">
+      <c r="J12" s="302">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),76,150,224,298,372,446,520,594,668,742,816,890)),"")</f>
         <v/>
       </c>
@@ -2671,25 +3167,25 @@
       <c r="N12" s="38" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="271">
+      <c r="A13" s="297">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),11,87,161,235,309,383,457,531,605,679,753,827))/INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),58,132,206,280,354,428,502,576,650,724,798,872)),"")</f>
         <v/>
       </c>
       <c r="B13" s="45" t="n"/>
       <c r="C13" s="46" t="n"/>
-      <c r="D13" s="278">
+      <c r="D13" s="305">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),31,105,179,253,327,401,475,549,623,697,771,845))/INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),58,132,206,280,354,428,502,576,650,724,798,872)),"")</f>
         <v/>
       </c>
       <c r="E13" s="45" t="n"/>
       <c r="F13" s="46" t="n"/>
-      <c r="G13" s="279">
+      <c r="G13" s="306">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),1,141,215,289,363,437,511,585,659,733,807,881))/INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),58,132,206,280,354,428,502,576,650,724,798,872)),"")</f>
         <v/>
       </c>
       <c r="H13" s="45" t="n"/>
       <c r="I13" s="46" t="n"/>
-      <c r="J13" s="280">
+      <c r="J13" s="307">
         <f>IFERROR(INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),76,150,224,298,372,446,520,594,668,742,816,890))/INDIRECT("'ESTADISTICA 2026'!B"&amp;CHOOSE(MATCH($C$5,{"ENERO","FEBRERO","MARZO","ABRIL","MAYO","JUNIO","JULIO","AGOSTO","SEPTIEMBRE","OCTUBRE","NOVIEMBRE","DICIEMBRE"},0),58,132,206,280,354,428,502,576,650,724,798,872)),"")</f>
         <v/>
       </c>
@@ -2716,19 +3212,19 @@
     </row>
     <row r="15" ht="8" customHeight="1">
       <c r="A15" s="238" t="n"/>
-      <c r="B15" s="238" t="n"/>
-      <c r="C15" s="238" t="n"/>
-      <c r="D15" s="238" t="n"/>
-      <c r="E15" s="238" t="n"/>
-      <c r="F15" s="238" t="n"/>
-      <c r="G15" s="238" t="n"/>
-      <c r="H15" s="238" t="n"/>
-      <c r="I15" s="238" t="n"/>
-      <c r="J15" s="238" t="n"/>
-      <c r="K15" s="238" t="n"/>
-      <c r="L15" s="238" t="n"/>
-      <c r="M15" s="238" t="n"/>
-      <c r="N15" s="238" t="n"/>
+      <c r="B15" s="45" t="n"/>
+      <c r="C15" s="45" t="n"/>
+      <c r="D15" s="45" t="n"/>
+      <c r="E15" s="45" t="n"/>
+      <c r="F15" s="45" t="n"/>
+      <c r="G15" s="45" t="n"/>
+      <c r="H15" s="45" t="n"/>
+      <c r="I15" s="45" t="n"/>
+      <c r="J15" s="45" t="n"/>
+      <c r="K15" s="45" t="n"/>
+      <c r="L15" s="45" t="n"/>
+      <c r="M15" s="45" t="n"/>
+      <c r="N15" s="46" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="113" t="inlineStr">
@@ -2979,356 +3475,364 @@
       <c r="N24" s="46" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="133" t="inlineStr">
+      <c r="A25" s="290" t="inlineStr">
         <is>
           <t>COBRANZA CORRIENTE</t>
         </is>
       </c>
-      <c r="E25" s="134" t="inlineStr">
+      <c r="B25" s="308" t="n"/>
+      <c r="C25" s="308" t="n"/>
+      <c r="E25" s="309" t="inlineStr">
         <is>
           <t>CANCELACIONES</t>
         </is>
       </c>
-      <c r="I25" s="135" t="inlineStr">
+      <c r="F25" s="310" t="n"/>
+      <c r="G25" s="310" t="n"/>
+      <c r="I25" s="311" t="inlineStr">
         <is>
           <t>COBRANZA VENCIDA</t>
         </is>
       </c>
-      <c r="M25" s="136" t="inlineStr">
+      <c r="J25" s="312" t="n"/>
+      <c r="K25" s="312" t="n"/>
+      <c r="M25" s="313" t="inlineStr">
         <is>
           <t>COBRANZA EFECTIVA</t>
         </is>
       </c>
+      <c r="N25" s="314" t="n"/>
+      <c r="O25" s="314" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="137" t="inlineStr">
+      <c r="A26" s="315" t="inlineStr">
         <is>
           <t>LUGAR</t>
         </is>
       </c>
-      <c r="B26" s="137" t="inlineStr">
+      <c r="B26" s="315" t="inlineStr">
         <is>
           <t>VENDEDOR</t>
         </is>
       </c>
-      <c r="C26" s="137" t="inlineStr">
+      <c r="C26" s="315" t="inlineStr">
         <is>
           <t>MONTO</t>
         </is>
       </c>
-      <c r="E26" s="138" t="inlineStr">
+      <c r="E26" s="315" t="inlineStr">
         <is>
           <t>LUGAR</t>
         </is>
       </c>
-      <c r="F26" s="138" t="inlineStr">
+      <c r="F26" s="315" t="inlineStr">
         <is>
           <t>VENDEDOR</t>
         </is>
       </c>
-      <c r="G26" s="138" t="inlineStr">
+      <c r="G26" s="315" t="inlineStr">
         <is>
           <t>MONTO</t>
         </is>
       </c>
-      <c r="I26" s="139" t="inlineStr">
+      <c r="I26" s="315" t="inlineStr">
         <is>
           <t>LUGAR</t>
         </is>
       </c>
-      <c r="J26" s="139" t="inlineStr">
+      <c r="J26" s="315" t="inlineStr">
         <is>
           <t>VENDEDOR</t>
         </is>
       </c>
-      <c r="K26" s="139" t="inlineStr">
+      <c r="K26" s="315" t="inlineStr">
         <is>
           <t>MONTO</t>
         </is>
       </c>
-      <c r="M26" s="140" t="inlineStr">
+      <c r="M26" s="315" t="inlineStr">
         <is>
           <t>LUGAR</t>
         </is>
       </c>
-      <c r="N26" s="140" t="inlineStr">
+      <c r="N26" s="315" t="inlineStr">
         <is>
           <t>VENDEDOR</t>
         </is>
       </c>
-      <c r="O26" s="140" t="inlineStr">
+      <c r="O26" s="315" t="inlineStr">
         <is>
           <t>MONTO</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="141" t="inlineStr">
+      <c r="A27" s="316" t="inlineStr">
         <is>
           <t>1er</t>
         </is>
       </c>
-      <c r="B27" s="142" t="inlineStr">
+      <c r="B27" s="317" t="inlineStr">
         <is>
           <t>V6</t>
         </is>
       </c>
-      <c r="C27" s="143" t="n">
+      <c r="C27" s="318" t="n">
         <v>356324</v>
       </c>
-      <c r="E27" s="144" t="inlineStr">
+      <c r="E27" s="316" t="inlineStr">
         <is>
           <t>1er</t>
         </is>
       </c>
-      <c r="F27" s="145" t="inlineStr">
+      <c r="F27" s="319" t="inlineStr">
         <is>
           <t>V38</t>
         </is>
       </c>
-      <c r="G27" s="146" t="n">
+      <c r="G27" s="318" t="n">
         <v>21035</v>
       </c>
-      <c r="I27" s="147" t="inlineStr">
+      <c r="I27" s="316" t="inlineStr">
         <is>
           <t>1er</t>
         </is>
       </c>
-      <c r="J27" s="148" t="inlineStr">
+      <c r="J27" s="320" t="inlineStr">
         <is>
           <t>V39 JOSE</t>
         </is>
       </c>
-      <c r="K27" s="149" t="n">
+      <c r="K27" s="318" t="n">
         <v>70796.5</v>
       </c>
-      <c r="M27" s="150" t="inlineStr">
+      <c r="M27" s="316" t="inlineStr">
         <is>
           <t>1er</t>
         </is>
       </c>
-      <c r="N27" s="151" t="inlineStr">
+      <c r="N27" s="321" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
       </c>
-      <c r="O27" s="152" t="n">
+      <c r="O27" s="318" t="n">
         <v>150839</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="153" t="inlineStr">
+      <c r="A28" s="322" t="inlineStr">
         <is>
           <t>2o</t>
         </is>
       </c>
-      <c r="B28" s="154" t="inlineStr">
+      <c r="B28" s="323" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="C28" s="155" t="n">
+      <c r="C28" s="324" t="n">
         <v>297307</v>
       </c>
-      <c r="E28" s="153" t="inlineStr">
+      <c r="E28" s="322" t="inlineStr">
         <is>
           <t>2o</t>
         </is>
       </c>
-      <c r="F28" s="154" t="inlineStr">
+      <c r="F28" s="325" t="inlineStr">
         <is>
           <t>V56</t>
         </is>
       </c>
-      <c r="G28" s="155" t="n">
+      <c r="G28" s="324" t="n">
         <v>17664</v>
       </c>
-      <c r="I28" s="153" t="inlineStr">
+      <c r="I28" s="322" t="inlineStr">
         <is>
           <t>2o</t>
         </is>
       </c>
-      <c r="J28" s="154" t="inlineStr">
+      <c r="J28" s="326" t="inlineStr">
         <is>
           <t>JORGE</t>
         </is>
       </c>
-      <c r="K28" s="155" t="n">
+      <c r="K28" s="324" t="n">
         <v>40169</v>
       </c>
-      <c r="M28" s="153" t="inlineStr">
+      <c r="M28" s="322" t="inlineStr">
         <is>
           <t>2o</t>
         </is>
       </c>
-      <c r="N28" s="154" t="inlineStr">
+      <c r="N28" s="327" t="inlineStr">
         <is>
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="O28" s="155" t="n">
+      <c r="O28" s="324" t="n">
         <v>140739</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="141" t="inlineStr">
+      <c r="A29" s="316" t="inlineStr">
         <is>
           <t>3o</t>
         </is>
       </c>
-      <c r="B29" s="142" t="inlineStr">
+      <c r="B29" s="317" t="inlineStr">
         <is>
           <t>V38</t>
         </is>
       </c>
-      <c r="C29" s="143" t="n">
+      <c r="C29" s="318" t="n">
         <v>241116</v>
       </c>
-      <c r="E29" s="144" t="inlineStr">
+      <c r="E29" s="316" t="inlineStr">
         <is>
           <t>3o</t>
         </is>
       </c>
-      <c r="F29" s="145" t="inlineStr">
+      <c r="F29" s="319" t="inlineStr">
         <is>
           <t>V6</t>
         </is>
       </c>
-      <c r="G29" s="146" t="n">
+      <c r="G29" s="318" t="n">
         <v>15924</v>
       </c>
-      <c r="I29" s="147" t="inlineStr">
+      <c r="I29" s="316" t="inlineStr">
         <is>
           <t>3er</t>
         </is>
       </c>
-      <c r="J29" s="148" t="inlineStr">
+      <c r="J29" s="320" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
       </c>
-      <c r="K29" s="149" t="n">
+      <c r="K29" s="318" t="n">
         <v>35046</v>
       </c>
-      <c r="M29" s="150" t="inlineStr">
+      <c r="M29" s="316" t="inlineStr">
         <is>
           <t>3o</t>
         </is>
       </c>
-      <c r="N29" s="151" t="inlineStr">
+      <c r="N29" s="321" t="inlineStr">
         <is>
           <t>EDUARDO</t>
         </is>
       </c>
-      <c r="O29" s="152" t="n">
+      <c r="O29" s="318" t="n">
         <v>91742</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="153" t="inlineStr">
+      <c r="A30" s="322" t="inlineStr">
         <is>
           <t>4o</t>
         </is>
       </c>
-      <c r="B30" s="154" t="inlineStr">
+      <c r="B30" s="323" t="inlineStr">
         <is>
           <t>V39</t>
         </is>
       </c>
-      <c r="C30" s="155" t="n">
+      <c r="C30" s="324" t="n">
         <v>176093</v>
       </c>
-      <c r="E30" s="153" t="inlineStr">
+      <c r="E30" s="322" t="inlineStr">
         <is>
           <t>4o</t>
         </is>
       </c>
-      <c r="F30" s="154" t="inlineStr">
+      <c r="F30" s="325" t="inlineStr">
         <is>
           <t>V84</t>
         </is>
       </c>
-      <c r="G30" s="155" t="n">
+      <c r="G30" s="324" t="n">
         <v>14374</v>
       </c>
-      <c r="I30" s="153" t="inlineStr">
+      <c r="I30" s="322" t="inlineStr">
         <is>
           <t>4o</t>
         </is>
       </c>
-      <c r="J30" s="154" t="inlineStr">
+      <c r="J30" s="326" t="inlineStr">
         <is>
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="K30" s="155" t="n">
+      <c r="K30" s="324" t="n">
         <v>34647</v>
       </c>
-      <c r="M30" s="153" t="inlineStr">
+      <c r="M30" s="322" t="inlineStr">
         <is>
           <t>4o</t>
         </is>
       </c>
-      <c r="N30" s="154" t="inlineStr">
+      <c r="N30" s="327" t="inlineStr">
         <is>
           <t>JORGE</t>
         </is>
       </c>
-      <c r="O30" s="155" t="n">
+      <c r="O30" s="324" t="n">
         <v>88710</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="141" t="inlineStr">
+      <c r="A31" s="316" t="inlineStr">
         <is>
           <t>5o</t>
         </is>
       </c>
-      <c r="B31" s="142" t="inlineStr">
+      <c r="B31" s="317" t="inlineStr">
         <is>
           <t>V56</t>
         </is>
       </c>
-      <c r="C31" s="143" t="n">
+      <c r="C31" s="318" t="n">
         <v>130775</v>
       </c>
-      <c r="E31" s="144" t="inlineStr">
+      <c r="E31" s="316" t="inlineStr">
         <is>
           <t>5o</t>
         </is>
       </c>
-      <c r="F31" s="145" t="inlineStr">
+      <c r="F31" s="319" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="G31" s="146" t="n">
+      <c r="G31" s="318" t="n">
         <v>13188</v>
       </c>
-      <c r="I31" s="147" t="inlineStr">
+      <c r="I31" s="316" t="inlineStr">
         <is>
           <t>5o</t>
         </is>
       </c>
-      <c r="J31" s="148" t="inlineStr">
+      <c r="J31" s="320" t="inlineStr">
         <is>
           <t>DEPOSITO</t>
         </is>
       </c>
-      <c r="K31" s="149" t="n">
+      <c r="K31" s="318" t="n">
         <v>24103.81</v>
       </c>
-      <c r="M31" s="150" t="inlineStr">
+      <c r="M31" s="316" t="inlineStr">
         <is>
           <t>5o</t>
         </is>
       </c>
-      <c r="N31" s="151" t="inlineStr">
+      <c r="N31" s="321" t="inlineStr">
         <is>
           <t>OFICINA</t>
         </is>
       </c>
-      <c r="O31" s="152" t="n">
+      <c r="O31" s="318" t="n">
         <v>28000</v>
       </c>
     </row>
@@ -3448,13 +3952,14 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="40">
+  <mergeCells count="41">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="D13:F13"/>
     <mergeCell ref="G13:I13"/>
     <mergeCell ref="A24:N24"/>
     <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A15:N15"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="M25:O25"/>
     <mergeCell ref="D7:F7"/>
@@ -3828,19 +4333,19 @@
   <dimension ref="A1:P914"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -5428,11 +5933,23 @@
     </row>
     <row r="78" ht="14" customHeight="1"/>
     <row r="79" ht="22" customHeight="1">
-      <c r="A79" s="4" t="inlineStr">
+      <c r="A79" s="328" t="inlineStr">
         <is>
           <t>FEBRERO 2026</t>
         </is>
       </c>
+      <c r="B79" s="329" t="n"/>
+      <c r="C79" s="329" t="n"/>
+      <c r="D79" s="329" t="n"/>
+      <c r="E79" s="329" t="n"/>
+      <c r="F79" s="329" t="n"/>
+      <c r="G79" s="329" t="n"/>
+      <c r="H79" s="329" t="n"/>
+      <c r="I79" s="329" t="n"/>
+      <c r="J79" s="329" t="n"/>
+      <c r="K79" s="329" t="n"/>
+      <c r="L79" s="329" t="n"/>
+      <c r="M79" s="329" t="n"/>
     </row>
     <row r="80" ht="28" customHeight="1">
       <c r="A80" s="5" t="inlineStr">
@@ -5573,462 +6090,495 @@
     </row>
     <row r="85" ht="6" customHeight="1"/>
     <row r="86">
-      <c r="A86" s="35" t="inlineStr">
+      <c r="A86" s="330" t="inlineStr">
         <is>
           <t>COBRANZA CORRIENTE</t>
         </is>
       </c>
-      <c r="B86" s="28" t="n"/>
-      <c r="C86" s="28" t="n"/>
-      <c r="D86" s="28" t="n"/>
-      <c r="E86" s="28" t="n"/>
-      <c r="F86" s="28" t="n"/>
-      <c r="G86" s="28" t="n"/>
-      <c r="H86" s="28" t="n"/>
-      <c r="I86" s="28" t="n"/>
-      <c r="J86" s="28" t="n"/>
-      <c r="K86" s="28" t="n"/>
-      <c r="L86" s="28" t="n"/>
-      <c r="M86" s="28" t="n"/>
+      <c r="B86" s="331" t="n"/>
+      <c r="C86" s="331" t="n"/>
+      <c r="D86" s="331" t="n"/>
+      <c r="E86" s="331" t="n"/>
+      <c r="F86" s="331" t="n"/>
+      <c r="G86" s="331" t="n"/>
+      <c r="H86" s="331" t="n"/>
+      <c r="I86" s="331" t="n"/>
+      <c r="J86" s="331" t="n"/>
+      <c r="K86" s="331" t="n"/>
+      <c r="L86" s="331" t="n"/>
+      <c r="M86" s="331" t="n"/>
       <c r="N86" s="28" t="n"/>
     </row>
     <row r="87" ht="20" customHeight="1">
-      <c r="A87" s="8" t="inlineStr">
+      <c r="A87" s="332" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B87" s="11" t="n">
+      <c r="B87" s="333" t="n">
         <v>1524936</v>
       </c>
+      <c r="C87" s="334" t="n"/>
+      <c r="D87" s="334" t="n"/>
+      <c r="E87" s="334" t="n"/>
+      <c r="F87" s="334" t="n"/>
+      <c r="G87" s="334" t="n"/>
+      <c r="H87" s="334" t="n"/>
+      <c r="I87" s="334" t="n"/>
+      <c r="J87" s="334" t="n"/>
+      <c r="K87" s="334" t="n"/>
+      <c r="L87" s="334" t="n"/>
+      <c r="M87" s="334" t="n"/>
     </row>
     <row r="88" ht="18" customHeight="1">
-      <c r="A88" s="12" t="inlineStr">
+      <c r="A88" s="335" t="inlineStr">
         <is>
           <t>Top 5</t>
         </is>
       </c>
-      <c r="C88" s="13" t="n"/>
-      <c r="D88" s="13" t="n"/>
-      <c r="E88" s="13" t="n"/>
-      <c r="F88" s="13" t="n"/>
-      <c r="G88" s="13" t="n"/>
-      <c r="H88" s="13" t="n"/>
-      <c r="I88" s="13" t="n"/>
-      <c r="J88" s="13" t="n"/>
-      <c r="K88" s="13" t="n"/>
-      <c r="L88" s="13" t="n"/>
-      <c r="M88" s="13" t="n"/>
+      <c r="C88" s="336" t="n"/>
+      <c r="D88" s="336" t="n"/>
+      <c r="E88" s="336" t="n"/>
+      <c r="F88" s="336" t="n"/>
+      <c r="G88" s="336" t="n"/>
+      <c r="H88" s="336" t="n"/>
+      <c r="I88" s="336" t="n"/>
+      <c r="J88" s="336" t="n"/>
+      <c r="K88" s="336" t="n"/>
+      <c r="L88" s="336" t="n"/>
+      <c r="M88" s="336" t="n"/>
       <c r="N88" s="13" t="n"/>
     </row>
     <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="14" t="inlineStr">
-        <is>
-          <t>1er lugar</t>
-        </is>
-      </c>
-      <c r="B89" s="15" t="n"/>
-      <c r="C89" s="15" t="inlineStr">
+      <c r="A89" s="337" t="inlineStr">
+        <is>
+          <t>1er</t>
+        </is>
+      </c>
+      <c r="B89" s="338" t="n"/>
+      <c r="C89" s="339" t="inlineStr">
         <is>
           <t>V6</t>
         </is>
       </c>
-      <c r="D89" s="15" t="n">
+      <c r="D89" s="340" t="n">
         <v>356324</v>
       </c>
-      <c r="E89" s="15" t="inlineStr">
+      <c r="E89" s="26" t="n"/>
+      <c r="F89" s="26" t="n"/>
+      <c r="G89" s="26" t="n"/>
+      <c r="H89" s="26" t="n"/>
+      <c r="I89" s="26" t="n"/>
+      <c r="J89" s="26" t="n"/>
+      <c r="K89" s="26" t="n"/>
+      <c r="L89" s="26" t="n"/>
+      <c r="M89" s="26" t="n"/>
+      <c r="N89" s="15" t="n"/>
+    </row>
+    <row r="90" ht="18" customHeight="1">
+      <c r="A90" s="341" t="inlineStr">
+        <is>
+          <t>2o</t>
+        </is>
+      </c>
+      <c r="B90" s="342" t="n"/>
+      <c r="C90" s="343" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="F89" s="15" t="n">
+      <c r="D90" s="344" t="n">
         <v>297307</v>
       </c>
-      <c r="G89" s="15" t="inlineStr">
+      <c r="E90" s="345" t="n"/>
+      <c r="F90" s="345" t="n"/>
+      <c r="G90" s="345" t="n"/>
+      <c r="H90" s="345" t="n"/>
+      <c r="I90" s="345" t="n"/>
+      <c r="J90" s="345" t="n"/>
+      <c r="K90" s="345" t="n"/>
+      <c r="L90" s="345" t="n"/>
+      <c r="M90" s="345" t="n"/>
+      <c r="N90" s="15" t="n"/>
+    </row>
+    <row r="91" ht="18" customHeight="1">
+      <c r="A91" s="337" t="inlineStr">
+        <is>
+          <t>3er</t>
+        </is>
+      </c>
+      <c r="B91" s="338" t="n"/>
+      <c r="C91" s="339" t="inlineStr">
         <is>
           <t>V38</t>
         </is>
       </c>
-      <c r="H89" s="15" t="n">
+      <c r="D91" s="340" t="n">
         <v>241116</v>
       </c>
-      <c r="I89" s="15" t="inlineStr">
+      <c r="E91" s="26" t="n"/>
+      <c r="F91" s="26" t="n"/>
+      <c r="G91" s="26" t="n"/>
+      <c r="H91" s="26" t="n"/>
+      <c r="I91" s="26" t="n"/>
+      <c r="J91" s="26" t="n"/>
+      <c r="K91" s="26" t="n"/>
+      <c r="L91" s="26" t="n"/>
+      <c r="M91" s="26" t="n"/>
+      <c r="N91" s="15" t="n"/>
+    </row>
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="341" t="inlineStr">
+        <is>
+          <t>4o</t>
+        </is>
+      </c>
+      <c r="B92" s="342" t="n"/>
+      <c r="C92" s="343" t="inlineStr">
         <is>
           <t>V39</t>
         </is>
       </c>
-      <c r="J89" s="15" t="n">
+      <c r="D92" s="344" t="n">
         <v>176093</v>
       </c>
-      <c r="K89" s="15" t="inlineStr">
+      <c r="E92" s="345" t="n"/>
+      <c r="F92" s="345" t="n"/>
+      <c r="G92" s="345" t="n"/>
+      <c r="H92" s="345" t="n"/>
+      <c r="I92" s="345" t="n"/>
+      <c r="J92" s="345" t="n"/>
+      <c r="K92" s="345" t="n"/>
+      <c r="L92" s="345" t="n"/>
+      <c r="M92" s="345" t="n"/>
+      <c r="N92" s="15" t="n"/>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="337" t="inlineStr">
+        <is>
+          <t>5o</t>
+        </is>
+      </c>
+      <c r="B93" s="338" t="n"/>
+      <c r="C93" s="339" t="inlineStr">
         <is>
           <t>V56</t>
         </is>
       </c>
-      <c r="L89" s="15" t="n">
+      <c r="D93" s="340" t="n">
         <v>130775</v>
       </c>
-      <c r="M89" s="15" t="n"/>
-      <c r="N89" s="15" t="n"/>
-    </row>
-    <row r="90" ht="18" customHeight="1">
-      <c r="A90" s="14" t="inlineStr">
-        <is>
-          <t>2o lugar</t>
-        </is>
-      </c>
-      <c r="B90" s="15" t="n"/>
-      <c r="C90" s="15" t="n"/>
-      <c r="D90" s="15" t="n"/>
-      <c r="E90" s="15" t="n"/>
-      <c r="F90" s="15" t="n"/>
-      <c r="G90" s="15" t="n"/>
-      <c r="H90" s="15" t="n"/>
-      <c r="I90" s="15" t="n"/>
-      <c r="J90" s="15" t="n"/>
-      <c r="K90" s="15" t="n"/>
-      <c r="L90" s="15" t="n"/>
-      <c r="M90" s="15" t="n"/>
-      <c r="N90" s="15" t="n"/>
-    </row>
-    <row r="91" ht="18" customHeight="1">
-      <c r="A91" s="14" t="inlineStr">
-        <is>
-          <t>3er lugar</t>
-        </is>
-      </c>
-      <c r="B91" s="15" t="n"/>
-      <c r="C91" s="15" t="n"/>
-      <c r="D91" s="15" t="n"/>
-      <c r="E91" s="15" t="n"/>
-      <c r="F91" s="15" t="n"/>
-      <c r="G91" s="15" t="n"/>
-      <c r="H91" s="15" t="n"/>
-      <c r="I91" s="15" t="n"/>
-      <c r="J91" s="15" t="n"/>
-      <c r="K91" s="15" t="n"/>
-      <c r="L91" s="15" t="n"/>
-      <c r="M91" s="15" t="n"/>
-      <c r="N91" s="15" t="n"/>
-    </row>
-    <row r="92" ht="18" customHeight="1">
-      <c r="A92" s="14" t="inlineStr">
-        <is>
-          <t>4o lugar</t>
-        </is>
-      </c>
-      <c r="B92" s="15" t="n"/>
-      <c r="C92" s="15" t="n"/>
-      <c r="D92" s="15" t="n"/>
-      <c r="E92" s="15" t="n"/>
-      <c r="F92" s="15" t="n"/>
-      <c r="G92" s="15" t="n"/>
-      <c r="H92" s="15" t="n"/>
-      <c r="I92" s="15" t="n"/>
-      <c r="J92" s="15" t="n"/>
-      <c r="K92" s="15" t="n"/>
-      <c r="L92" s="15" t="n"/>
-      <c r="M92" s="15" t="n"/>
-      <c r="N92" s="15" t="n"/>
-    </row>
-    <row r="93" ht="18" customHeight="1">
-      <c r="A93" s="14" t="inlineStr">
-        <is>
-          <t>5o lugar</t>
-        </is>
-      </c>
-      <c r="B93" s="15" t="n"/>
-      <c r="C93" s="15" t="n"/>
-      <c r="D93" s="15" t="n"/>
-      <c r="E93" s="15" t="n"/>
-      <c r="F93" s="15" t="n"/>
-      <c r="G93" s="15" t="n"/>
-      <c r="H93" s="15" t="n"/>
-      <c r="I93" s="15" t="n"/>
-      <c r="J93" s="15" t="n"/>
-      <c r="K93" s="15" t="n"/>
-      <c r="L93" s="15" t="n"/>
-      <c r="M93" s="15" t="n"/>
+      <c r="E93" s="26" t="n"/>
+      <c r="F93" s="26" t="n"/>
+      <c r="G93" s="26" t="n"/>
+      <c r="H93" s="26" t="n"/>
+      <c r="I93" s="26" t="n"/>
+      <c r="J93" s="26" t="n"/>
+      <c r="K93" s="26" t="n"/>
+      <c r="L93" s="26" t="n"/>
+      <c r="M93" s="26" t="n"/>
       <c r="N93" s="15" t="n"/>
     </row>
     <row r="94" ht="6" customHeight="1"/>
     <row r="95">
-      <c r="A95" s="35" t="inlineStr">
+      <c r="A95" s="346" t="inlineStr">
         <is>
           <t>CANCELACIONES</t>
         </is>
       </c>
-      <c r="B95" s="28" t="n"/>
-      <c r="C95" s="28" t="n"/>
-      <c r="D95" s="28" t="n"/>
-      <c r="E95" s="28" t="n"/>
-      <c r="F95" s="28" t="n"/>
-      <c r="G95" s="28" t="n"/>
-      <c r="H95" s="28" t="n"/>
-      <c r="I95" s="28" t="n"/>
-      <c r="J95" s="28" t="n"/>
-      <c r="K95" s="28" t="n"/>
-      <c r="L95" s="28" t="n"/>
-      <c r="M95" s="28" t="n"/>
+      <c r="B95" s="347" t="n"/>
+      <c r="C95" s="347" t="n"/>
+      <c r="D95" s="347" t="n"/>
+      <c r="E95" s="347" t="n"/>
+      <c r="F95" s="347" t="n"/>
+      <c r="G95" s="347" t="n"/>
+      <c r="H95" s="347" t="n"/>
+      <c r="I95" s="347" t="n"/>
+      <c r="J95" s="347" t="n"/>
+      <c r="K95" s="347" t="n"/>
+      <c r="L95" s="347" t="n"/>
+      <c r="M95" s="347" t="n"/>
       <c r="N95" s="28" t="n"/>
     </row>
     <row r="96" ht="20" customHeight="1">
-      <c r="A96" s="16" t="inlineStr">
+      <c r="A96" s="348" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B96" s="17" t="n">
+      <c r="B96" s="349" t="n">
         <v>174435</v>
       </c>
+      <c r="C96" s="350" t="n"/>
+      <c r="D96" s="350" t="n"/>
+      <c r="E96" s="350" t="n"/>
+      <c r="F96" s="350" t="n"/>
+      <c r="G96" s="350" t="n"/>
+      <c r="H96" s="350" t="n"/>
+      <c r="I96" s="350" t="n"/>
+      <c r="J96" s="350" t="n"/>
+      <c r="K96" s="350" t="n"/>
+      <c r="L96" s="350" t="n"/>
+      <c r="M96" s="350" t="n"/>
     </row>
     <row r="97" ht="18" customHeight="1">
-      <c r="A97" s="12" t="inlineStr">
+      <c r="A97" s="335" t="inlineStr">
         <is>
           <t>Top 5</t>
         </is>
       </c>
-      <c r="C97" s="13" t="n"/>
-      <c r="D97" s="13" t="n"/>
-      <c r="E97" s="13" t="n"/>
-      <c r="F97" s="13" t="n"/>
-      <c r="G97" s="13" t="n"/>
-      <c r="H97" s="13" t="n"/>
-      <c r="I97" s="13" t="n"/>
-      <c r="J97" s="13" t="n"/>
-      <c r="K97" s="13" t="n"/>
-      <c r="L97" s="13" t="n"/>
-      <c r="M97" s="13" t="n"/>
+      <c r="C97" s="336" t="n"/>
+      <c r="D97" s="336" t="n"/>
+      <c r="E97" s="336" t="n"/>
+      <c r="F97" s="336" t="n"/>
+      <c r="G97" s="336" t="n"/>
+      <c r="H97" s="336" t="n"/>
+      <c r="I97" s="336" t="n"/>
+      <c r="J97" s="336" t="n"/>
+      <c r="K97" s="336" t="n"/>
+      <c r="L97" s="336" t="n"/>
+      <c r="M97" s="336" t="n"/>
       <c r="N97" s="13" t="n"/>
     </row>
     <row r="98" ht="18" customHeight="1">
-      <c r="A98" s="14" t="inlineStr">
-        <is>
-          <t>1er lugar</t>
-        </is>
-      </c>
-      <c r="B98" s="15" t="n"/>
-      <c r="C98" s="15" t="inlineStr">
+      <c r="A98" s="337" t="inlineStr">
+        <is>
+          <t>1er</t>
+        </is>
+      </c>
+      <c r="B98" s="338" t="n"/>
+      <c r="C98" s="351" t="inlineStr">
         <is>
           <t>V38</t>
         </is>
       </c>
-      <c r="D98" s="15" t="n">
+      <c r="D98" s="340" t="n">
         <v>21035</v>
       </c>
-      <c r="E98" s="15" t="inlineStr">
+      <c r="E98" s="26" t="n"/>
+      <c r="F98" s="26" t="n"/>
+      <c r="G98" s="26" t="n"/>
+      <c r="H98" s="26" t="n"/>
+      <c r="I98" s="26" t="n"/>
+      <c r="J98" s="26" t="n"/>
+      <c r="K98" s="26" t="n"/>
+      <c r="L98" s="26" t="n"/>
+      <c r="M98" s="26" t="n"/>
+      <c r="N98" s="15" t="n"/>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="341" t="inlineStr">
+        <is>
+          <t>2o</t>
+        </is>
+      </c>
+      <c r="B99" s="342" t="n"/>
+      <c r="C99" s="352" t="inlineStr">
         <is>
           <t>V56</t>
         </is>
       </c>
-      <c r="F98" s="15" t="n">
+      <c r="D99" s="344" t="n">
         <v>17664</v>
       </c>
-      <c r="G98" s="15" t="inlineStr">
+      <c r="E99" s="345" t="n"/>
+      <c r="F99" s="345" t="n"/>
+      <c r="G99" s="345" t="n"/>
+      <c r="H99" s="345" t="n"/>
+      <c r="I99" s="345" t="n"/>
+      <c r="J99" s="345" t="n"/>
+      <c r="K99" s="345" t="n"/>
+      <c r="L99" s="345" t="n"/>
+      <c r="M99" s="345" t="n"/>
+      <c r="N99" s="15" t="n"/>
+    </row>
+    <row r="100" ht="18" customHeight="1">
+      <c r="A100" s="337" t="inlineStr">
+        <is>
+          <t>3er</t>
+        </is>
+      </c>
+      <c r="B100" s="338" t="n"/>
+      <c r="C100" s="351" t="inlineStr">
         <is>
           <t>V6</t>
         </is>
       </c>
-      <c r="H98" s="15" t="n">
+      <c r="D100" s="340" t="n">
         <v>15924</v>
       </c>
-      <c r="I98" s="15" t="inlineStr">
+      <c r="E100" s="26" t="n"/>
+      <c r="F100" s="26" t="n"/>
+      <c r="G100" s="26" t="n"/>
+      <c r="H100" s="26" t="n"/>
+      <c r="I100" s="26" t="n"/>
+      <c r="J100" s="26" t="n"/>
+      <c r="K100" s="26" t="n"/>
+      <c r="L100" s="26" t="n"/>
+      <c r="M100" s="26" t="n"/>
+      <c r="N100" s="15" t="n"/>
+    </row>
+    <row r="101" ht="18" customHeight="1">
+      <c r="A101" s="341" t="inlineStr">
+        <is>
+          <t>4o</t>
+        </is>
+      </c>
+      <c r="B101" s="342" t="n"/>
+      <c r="C101" s="352" t="inlineStr">
         <is>
           <t>V84</t>
         </is>
       </c>
-      <c r="J98" s="15" t="n">
+      <c r="D101" s="344" t="n">
         <v>14374</v>
       </c>
-      <c r="K98" s="15" t="inlineStr">
+      <c r="E101" s="345" t="n"/>
+      <c r="F101" s="345" t="n"/>
+      <c r="G101" s="345" t="n"/>
+      <c r="H101" s="345" t="n"/>
+      <c r="I101" s="345" t="n"/>
+      <c r="J101" s="345" t="n"/>
+      <c r="K101" s="345" t="n"/>
+      <c r="L101" s="345" t="n"/>
+      <c r="M101" s="345" t="n"/>
+      <c r="N101" s="15" t="n"/>
+    </row>
+    <row r="102" ht="18" customHeight="1">
+      <c r="A102" s="337" t="inlineStr">
+        <is>
+          <t>5o</t>
+        </is>
+      </c>
+      <c r="B102" s="338" t="n"/>
+      <c r="C102" s="351" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="L98" s="15" t="n">
+      <c r="D102" s="340" t="n">
         <v>13188</v>
       </c>
-      <c r="M98" s="15" t="n"/>
-      <c r="N98" s="15" t="n"/>
-    </row>
-    <row r="99" ht="18" customHeight="1">
-      <c r="A99" s="14" t="inlineStr">
-        <is>
-          <t>2o lugar</t>
-        </is>
-      </c>
-      <c r="B99" s="15" t="n"/>
-      <c r="C99" s="15" t="n"/>
-      <c r="D99" s="15" t="n"/>
-      <c r="E99" s="15" t="n"/>
-      <c r="F99" s="15" t="n"/>
-      <c r="G99" s="15" t="n"/>
-      <c r="H99" s="15" t="n"/>
-      <c r="I99" s="15" t="n"/>
-      <c r="J99" s="15" t="n"/>
-      <c r="K99" s="15" t="n"/>
-      <c r="L99" s="15" t="n"/>
-      <c r="M99" s="15" t="n"/>
-      <c r="N99" s="15" t="n"/>
-    </row>
-    <row r="100" ht="18" customHeight="1">
-      <c r="A100" s="14" t="inlineStr">
-        <is>
-          <t>3er lugar</t>
-        </is>
-      </c>
-      <c r="B100" s="15" t="n"/>
-      <c r="C100" s="15" t="n"/>
-      <c r="D100" s="15" t="n"/>
-      <c r="E100" s="15" t="n"/>
-      <c r="F100" s="15" t="n"/>
-      <c r="G100" s="15" t="n"/>
-      <c r="H100" s="15" t="n"/>
-      <c r="I100" s="15" t="n"/>
-      <c r="J100" s="15" t="n"/>
-      <c r="K100" s="15" t="n"/>
-      <c r="L100" s="15" t="n"/>
-      <c r="M100" s="15" t="n"/>
-      <c r="N100" s="15" t="n"/>
-    </row>
-    <row r="101" ht="18" customHeight="1">
-      <c r="A101" s="14" t="inlineStr">
-        <is>
-          <t>4o lugar</t>
-        </is>
-      </c>
-      <c r="B101" s="15" t="n"/>
-      <c r="C101" s="15" t="n"/>
-      <c r="D101" s="15" t="n"/>
-      <c r="E101" s="15" t="n"/>
-      <c r="F101" s="15" t="n"/>
-      <c r="G101" s="15" t="n"/>
-      <c r="H101" s="15" t="n"/>
-      <c r="I101" s="15" t="n"/>
-      <c r="J101" s="15" t="n"/>
-      <c r="K101" s="15" t="n"/>
-      <c r="L101" s="15" t="n"/>
-      <c r="M101" s="15" t="n"/>
-      <c r="N101" s="15" t="n"/>
-    </row>
-    <row r="102" ht="18" customHeight="1">
-      <c r="A102" s="14" t="inlineStr">
-        <is>
-          <t>5o lugar</t>
-        </is>
-      </c>
-      <c r="B102" s="15" t="n"/>
-      <c r="C102" s="15" t="n"/>
-      <c r="D102" s="15" t="n"/>
-      <c r="E102" s="15" t="n"/>
-      <c r="F102" s="15" t="n"/>
-      <c r="G102" s="15" t="n"/>
-      <c r="H102" s="15" t="n"/>
-      <c r="I102" s="15" t="n"/>
-      <c r="J102" s="15" t="n"/>
-      <c r="K102" s="15" t="n"/>
-      <c r="L102" s="15" t="n"/>
-      <c r="M102" s="15" t="n"/>
+      <c r="E102" s="26" t="n"/>
+      <c r="F102" s="26" t="n"/>
+      <c r="G102" s="26" t="n"/>
+      <c r="H102" s="26" t="n"/>
+      <c r="I102" s="26" t="n"/>
+      <c r="J102" s="26" t="n"/>
+      <c r="K102" s="26" t="n"/>
+      <c r="L102" s="26" t="n"/>
+      <c r="M102" s="26" t="n"/>
       <c r="N102" s="15" t="n"/>
     </row>
     <row r="103" ht="6" customHeight="1"/>
     <row r="104">
-      <c r="A104" s="35" t="inlineStr">
+      <c r="A104" s="353" t="inlineStr">
         <is>
           <t>COBRANZA VENCIDA</t>
         </is>
       </c>
-      <c r="B104" s="28" t="n"/>
-      <c r="C104" s="28" t="n"/>
-      <c r="D104" s="28" t="n"/>
-      <c r="E104" s="28" t="n"/>
-      <c r="F104" s="28" t="n"/>
-      <c r="G104" s="28" t="n"/>
-      <c r="H104" s="28" t="n"/>
-      <c r="I104" s="28" t="n"/>
-      <c r="J104" s="28" t="n"/>
-      <c r="K104" s="28" t="n"/>
-      <c r="L104" s="28" t="n"/>
-      <c r="M104" s="28" t="n"/>
+      <c r="B104" s="354" t="n"/>
+      <c r="C104" s="354" t="n"/>
+      <c r="D104" s="354" t="n"/>
+      <c r="E104" s="354" t="n"/>
+      <c r="F104" s="354" t="n"/>
+      <c r="G104" s="354" t="n"/>
+      <c r="H104" s="354" t="n"/>
+      <c r="I104" s="354" t="n"/>
+      <c r="J104" s="354" t="n"/>
+      <c r="K104" s="354" t="n"/>
+      <c r="L104" s="354" t="n"/>
+      <c r="M104" s="354" t="n"/>
       <c r="N104" s="28" t="n"/>
     </row>
     <row r="105" ht="20" customHeight="1">
-      <c r="A105" s="8" t="inlineStr">
+      <c r="A105" s="355" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B105" s="11" t="n">
+      <c r="B105" s="356" t="n">
         <v>251487.31</v>
       </c>
+      <c r="C105" s="357" t="n"/>
+      <c r="D105" s="357" t="n"/>
+      <c r="E105" s="357" t="n"/>
+      <c r="F105" s="357" t="n"/>
+      <c r="G105" s="357" t="n"/>
+      <c r="H105" s="357" t="n"/>
+      <c r="I105" s="357" t="n"/>
+      <c r="J105" s="357" t="n"/>
+      <c r="K105" s="357" t="n"/>
+      <c r="L105" s="357" t="n"/>
+      <c r="M105" s="357" t="n"/>
     </row>
     <row r="106" ht="18" customHeight="1">
-      <c r="A106" s="12" t="inlineStr">
+      <c r="A106" s="335" t="inlineStr">
         <is>
           <t>Top 5</t>
         </is>
       </c>
-      <c r="C106" s="13" t="n"/>
-      <c r="D106" s="13" t="n"/>
-      <c r="E106" s="13" t="n"/>
-      <c r="F106" s="13" t="n"/>
-      <c r="G106" s="13" t="n"/>
-      <c r="H106" s="13" t="n"/>
-      <c r="I106" s="13" t="n"/>
-      <c r="J106" s="13" t="n"/>
-      <c r="K106" s="13" t="n"/>
-      <c r="L106" s="13" t="n"/>
-      <c r="M106" s="13" t="n"/>
+      <c r="C106" s="336" t="n"/>
+      <c r="D106" s="336" t="n"/>
+      <c r="E106" s="336" t="n"/>
+      <c r="F106" s="336" t="n"/>
+      <c r="G106" s="336" t="n"/>
+      <c r="H106" s="336" t="n"/>
+      <c r="I106" s="336" t="n"/>
+      <c r="J106" s="336" t="n"/>
+      <c r="K106" s="336" t="n"/>
+      <c r="L106" s="336" t="n"/>
+      <c r="M106" s="336" t="n"/>
       <c r="N106" s="13" t="n"/>
     </row>
     <row r="107" ht="18" customHeight="1">
-      <c r="A107" s="14" t="inlineStr">
-        <is>
-          <t>1er lugar</t>
-        </is>
-      </c>
-      <c r="B107" s="15" t="n"/>
-      <c r="C107" s="15" t="inlineStr">
+      <c r="A107" s="337" t="inlineStr">
+        <is>
+          <t>1er</t>
+        </is>
+      </c>
+      <c r="B107" s="338" t="n"/>
+      <c r="C107" s="358" t="inlineStr">
         <is>
           <t>V39 JOSE</t>
         </is>
       </c>
-      <c r="D107" s="15" t="n">
+      <c r="D107" s="340" t="n">
         <v>70796.5</v>
       </c>
-      <c r="E107" s="15" t="inlineStr">
+      <c r="E107" s="26" t="inlineStr">
         <is>
           <t>JORGE</t>
         </is>
       </c>
-      <c r="F107" s="15" t="n">
+      <c r="F107" s="26" t="n">
         <v>40169</v>
       </c>
-      <c r="G107" s="15" t="inlineStr">
+      <c r="G107" s="26" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
       </c>
-      <c r="H107" s="15" t="n">
+      <c r="H107" s="26" t="n">
         <v>35046</v>
       </c>
-      <c r="I107" s="15" t="inlineStr">
+      <c r="I107" s="26" t="inlineStr">
         <is>
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="J107" s="15" t="n">
+      <c r="J107" s="26" t="n">
         <v>34647</v>
       </c>
-      <c r="K107" s="15" t="inlineStr">
+      <c r="K107" s="26" t="inlineStr">
         <is>
           <t>DEPOSITO</t>
         </is>
       </c>
-      <c r="L107" s="15" t="n">
+      <c r="L107" s="26" t="n">
         <v>24103.81</v>
       </c>
-      <c r="M107" s="15" t="n">
+      <c r="M107" s="26" t="n">
         <v>0.2815</v>
       </c>
       <c r="N107" s="15" t="n">
@@ -6036,932 +6586,1036 @@
       </c>
     </row>
     <row r="108" ht="18" customHeight="1">
-      <c r="A108" s="14" t="inlineStr">
-        <is>
-          <t>2o lugar</t>
-        </is>
-      </c>
-      <c r="B108" s="15" t="n"/>
-      <c r="C108" s="15" t="n"/>
-      <c r="D108" s="15" t="n"/>
-      <c r="E108" s="15" t="inlineStr">
+      <c r="A108" s="341" t="inlineStr">
+        <is>
+          <t>2o</t>
+        </is>
+      </c>
+      <c r="B108" s="342" t="n"/>
+      <c r="C108" s="359" t="n"/>
+      <c r="D108" s="344" t="n"/>
+      <c r="E108" s="345" t="inlineStr">
         <is>
           <t>JORGE</t>
         </is>
       </c>
-      <c r="F108" s="15" t="n">
+      <c r="F108" s="345" t="n">
         <v>40169</v>
       </c>
-      <c r="G108" s="15" t="n"/>
-      <c r="H108" s="15" t="n"/>
-      <c r="I108" s="15" t="n"/>
-      <c r="J108" s="15" t="n"/>
-      <c r="K108" s="15" t="n"/>
-      <c r="L108" s="15" t="n"/>
-      <c r="M108" s="15" t="n">
-        <v>0.1597</v>
-      </c>
+      <c r="G108" s="345" t="n"/>
+      <c r="H108" s="345" t="n"/>
+      <c r="I108" s="345" t="n"/>
+      <c r="J108" s="345" t="n"/>
+      <c r="K108" s="345" t="n"/>
+      <c r="L108" s="345" t="n"/>
+      <c r="M108" s="345" t="n"/>
       <c r="N108" s="15" t="n">
         <v>0.4412</v>
       </c>
     </row>
     <row r="109" ht="18" customHeight="1">
-      <c r="A109" s="14" t="inlineStr">
-        <is>
-          <t>3er lugar</t>
-        </is>
-      </c>
-      <c r="B109" s="15" t="n"/>
-      <c r="C109" s="15" t="n"/>
-      <c r="D109" s="15" t="n"/>
-      <c r="E109" s="15" t="n"/>
-      <c r="F109" s="15" t="n"/>
-      <c r="G109" s="15" t="inlineStr">
+      <c r="A109" s="337" t="inlineStr">
+        <is>
+          <t>3er</t>
+        </is>
+      </c>
+      <c r="B109" s="338" t="n"/>
+      <c r="C109" s="358" t="n"/>
+      <c r="D109" s="340" t="n"/>
+      <c r="E109" s="26" t="n"/>
+      <c r="F109" s="26" t="n"/>
+      <c r="G109" s="26" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
       </c>
-      <c r="H109" s="15" t="n">
+      <c r="H109" s="26" t="n">
         <v>35046</v>
       </c>
-      <c r="I109" s="15" t="n"/>
-      <c r="J109" s="15" t="n"/>
-      <c r="K109" s="15" t="n"/>
-      <c r="L109" s="15" t="n"/>
-      <c r="M109" s="15" t="n">
-        <v>0.1394</v>
-      </c>
+      <c r="I109" s="26" t="n"/>
+      <c r="J109" s="26" t="n"/>
+      <c r="K109" s="26" t="n"/>
+      <c r="L109" s="26" t="n"/>
+      <c r="M109" s="26" t="n"/>
       <c r="N109" s="15" t="n">
         <v>0.5806</v>
       </c>
     </row>
     <row r="110" ht="18" customHeight="1">
-      <c r="A110" s="14" t="inlineStr">
-        <is>
-          <t>4o lugar</t>
-        </is>
-      </c>
-      <c r="B110" s="15" t="n"/>
-      <c r="C110" s="15" t="n"/>
-      <c r="D110" s="15" t="n"/>
-      <c r="E110" s="15" t="n"/>
-      <c r="F110" s="15" t="n"/>
-      <c r="G110" s="15" t="n"/>
-      <c r="H110" s="15" t="n"/>
-      <c r="I110" s="15" t="inlineStr">
+      <c r="A110" s="341" t="inlineStr">
+        <is>
+          <t>4o</t>
+        </is>
+      </c>
+      <c r="B110" s="342" t="n"/>
+      <c r="C110" s="359" t="n"/>
+      <c r="D110" s="344" t="n"/>
+      <c r="E110" s="345" t="n"/>
+      <c r="F110" s="345" t="n"/>
+      <c r="G110" s="345" t="n"/>
+      <c r="H110" s="345" t="n"/>
+      <c r="I110" s="345" t="inlineStr">
         <is>
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="J110" s="15" t="n">
+      <c r="J110" s="345" t="n">
         <v>34647</v>
       </c>
-      <c r="K110" s="15" t="n"/>
-      <c r="L110" s="15" t="n"/>
-      <c r="M110" s="15" t="n">
-        <v>0.1378</v>
-      </c>
+      <c r="K110" s="345" t="n"/>
+      <c r="L110" s="345" t="n"/>
+      <c r="M110" s="345" t="n"/>
       <c r="N110" s="15" t="n">
         <v>0.7184</v>
       </c>
     </row>
     <row r="111" ht="18" customHeight="1">
-      <c r="A111" s="14" t="inlineStr">
-        <is>
-          <t>5o lugar</t>
-        </is>
-      </c>
-      <c r="B111" s="15" t="n"/>
-      <c r="C111" s="15" t="n"/>
-      <c r="D111" s="15" t="n"/>
-      <c r="E111" s="15" t="n"/>
-      <c r="F111" s="15" t="n"/>
-      <c r="G111" s="15" t="n"/>
-      <c r="H111" s="15" t="n"/>
-      <c r="I111" s="15" t="n"/>
-      <c r="J111" s="15" t="n"/>
-      <c r="K111" s="15" t="inlineStr">
+      <c r="A111" s="337" t="inlineStr">
+        <is>
+          <t>5o</t>
+        </is>
+      </c>
+      <c r="B111" s="338" t="n"/>
+      <c r="C111" s="358" t="n"/>
+      <c r="D111" s="340" t="n"/>
+      <c r="E111" s="26" t="n"/>
+      <c r="F111" s="26" t="n"/>
+      <c r="G111" s="26" t="n"/>
+      <c r="H111" s="26" t="n"/>
+      <c r="I111" s="26" t="n"/>
+      <c r="J111" s="26" t="n"/>
+      <c r="K111" s="26" t="inlineStr">
         <is>
           <t>DEPOSITO</t>
         </is>
       </c>
-      <c r="L111" s="15" t="n">
+      <c r="L111" s="26" t="n">
         <v>24103.81</v>
       </c>
-      <c r="M111" s="15" t="n">
-        <v>0.0958</v>
-      </c>
+      <c r="M111" s="26" t="n"/>
       <c r="N111" s="15" t="n">
         <v>0.8142</v>
       </c>
     </row>
     <row r="112" ht="6" customHeight="1"/>
     <row r="113">
-      <c r="A113" s="35" t="inlineStr">
+      <c r="A113" s="360" t="inlineStr">
         <is>
           <t>COBRANZA EFECTIVA</t>
         </is>
       </c>
-      <c r="B113" s="28" t="n"/>
-      <c r="C113" s="28" t="n"/>
-      <c r="D113" s="28" t="n"/>
-      <c r="E113" s="28" t="n"/>
-      <c r="F113" s="28" t="n"/>
-      <c r="G113" s="28" t="n"/>
-      <c r="H113" s="28" t="n"/>
-      <c r="I113" s="28" t="n"/>
-      <c r="J113" s="28" t="n"/>
-      <c r="K113" s="28" t="n"/>
-      <c r="L113" s="28" t="n"/>
-      <c r="M113" s="28" t="n"/>
+      <c r="B113" s="361" t="n"/>
+      <c r="C113" s="361" t="n"/>
+      <c r="D113" s="361" t="n"/>
+      <c r="E113" s="361" t="n"/>
+      <c r="F113" s="361" t="n"/>
+      <c r="G113" s="361" t="n"/>
+      <c r="H113" s="361" t="n"/>
+      <c r="I113" s="361" t="n"/>
+      <c r="J113" s="361" t="n"/>
+      <c r="K113" s="361" t="n"/>
+      <c r="L113" s="361" t="n"/>
+      <c r="M113" s="361" t="n"/>
       <c r="N113" s="28" t="n"/>
     </row>
     <row r="114" ht="20" customHeight="1">
-      <c r="A114" s="16" t="inlineStr">
+      <c r="A114" s="362" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B114" s="17" t="n">
+      <c r="B114" s="363" t="n">
         <v>1110578</v>
       </c>
+      <c r="C114" s="364" t="n"/>
+      <c r="D114" s="364" t="n"/>
+      <c r="E114" s="364" t="n"/>
+      <c r="F114" s="364" t="n"/>
+      <c r="G114" s="364" t="n"/>
+      <c r="H114" s="364" t="n"/>
+      <c r="I114" s="364" t="n"/>
+      <c r="J114" s="364" t="n"/>
+      <c r="K114" s="364" t="n"/>
+      <c r="L114" s="364" t="n"/>
+      <c r="M114" s="364" t="n"/>
     </row>
     <row r="115" ht="18" customHeight="1">
-      <c r="A115" s="12" t="inlineStr">
+      <c r="A115" s="335" t="inlineStr">
         <is>
           <t>Top 5</t>
         </is>
       </c>
-      <c r="C115" s="13" t="n"/>
-      <c r="D115" s="13" t="n"/>
-      <c r="E115" s="13" t="n"/>
-      <c r="F115" s="13" t="n"/>
-      <c r="G115" s="13" t="n"/>
-      <c r="H115" s="13" t="n"/>
-      <c r="I115" s="13" t="n"/>
-      <c r="J115" s="13" t="n"/>
-      <c r="K115" s="13" t="n"/>
-      <c r="L115" s="13" t="n"/>
-      <c r="M115" s="13" t="n"/>
+      <c r="C115" s="336" t="n"/>
+      <c r="D115" s="336" t="n"/>
+      <c r="E115" s="336" t="n"/>
+      <c r="F115" s="336" t="n"/>
+      <c r="G115" s="336" t="n"/>
+      <c r="H115" s="336" t="n"/>
+      <c r="I115" s="336" t="n"/>
+      <c r="J115" s="336" t="n"/>
+      <c r="K115" s="336" t="n"/>
+      <c r="L115" s="336" t="n"/>
+      <c r="M115" s="336" t="n"/>
       <c r="N115" s="13" t="n"/>
     </row>
     <row r="116" ht="18" customHeight="1">
-      <c r="A116" s="14" t="inlineStr">
-        <is>
-          <t>1er lugar</t>
-        </is>
-      </c>
-      <c r="B116" s="15" t="n"/>
-      <c r="C116" s="15" t="inlineStr">
+      <c r="A116" s="337" t="inlineStr">
+        <is>
+          <t>1er</t>
+        </is>
+      </c>
+      <c r="B116" s="338" t="n"/>
+      <c r="C116" s="365" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
       </c>
-      <c r="D116" s="15" t="n">
+      <c r="D116" s="340" t="n">
         <v>150839</v>
       </c>
-      <c r="E116" s="15" t="inlineStr">
+      <c r="E116" s="26" t="n"/>
+      <c r="F116" s="26" t="n"/>
+      <c r="G116" s="26" t="n"/>
+      <c r="H116" s="26" t="n"/>
+      <c r="I116" s="26" t="n"/>
+      <c r="J116" s="26" t="n"/>
+      <c r="K116" s="26" t="n"/>
+      <c r="L116" s="26" t="n"/>
+      <c r="M116" s="26" t="n"/>
+      <c r="N116" s="15" t="n"/>
+    </row>
+    <row r="117" ht="18" customHeight="1">
+      <c r="A117" s="341" t="inlineStr">
+        <is>
+          <t>2o</t>
+        </is>
+      </c>
+      <c r="B117" s="342" t="n"/>
+      <c r="C117" s="366" t="inlineStr">
         <is>
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="F116" s="15" t="n">
+      <c r="D117" s="344" t="n">
         <v>140739</v>
       </c>
-      <c r="G116" s="15" t="inlineStr">
+      <c r="E117" s="345" t="n"/>
+      <c r="F117" s="345" t="n"/>
+      <c r="G117" s="345" t="n"/>
+      <c r="H117" s="345" t="n"/>
+      <c r="I117" s="345" t="n"/>
+      <c r="J117" s="345" t="n"/>
+      <c r="K117" s="345" t="n"/>
+      <c r="L117" s="345" t="n"/>
+      <c r="M117" s="345" t="n"/>
+      <c r="N117" s="15" t="n"/>
+    </row>
+    <row r="118" ht="18" customHeight="1">
+      <c r="A118" s="337" t="inlineStr">
+        <is>
+          <t>3er</t>
+        </is>
+      </c>
+      <c r="B118" s="338" t="n"/>
+      <c r="C118" s="365" t="inlineStr">
         <is>
           <t>EDUARDO</t>
         </is>
       </c>
-      <c r="H116" s="15" t="n">
+      <c r="D118" s="340" t="n">
         <v>91742</v>
       </c>
-      <c r="I116" s="15" t="inlineStr">
+      <c r="E118" s="26" t="n"/>
+      <c r="F118" s="26" t="n"/>
+      <c r="G118" s="26" t="n"/>
+      <c r="H118" s="26" t="n"/>
+      <c r="I118" s="26" t="n"/>
+      <c r="J118" s="26" t="n"/>
+      <c r="K118" s="26" t="n"/>
+      <c r="L118" s="26" t="n"/>
+      <c r="M118" s="26" t="n"/>
+      <c r="N118" s="15" t="n"/>
+    </row>
+    <row r="119" ht="18" customHeight="1">
+      <c r="A119" s="341" t="inlineStr">
+        <is>
+          <t>4o</t>
+        </is>
+      </c>
+      <c r="B119" s="342" t="n"/>
+      <c r="C119" s="366" t="inlineStr">
         <is>
           <t>JORGE</t>
         </is>
       </c>
-      <c r="J116" s="15" t="n">
+      <c r="D119" s="344" t="n">
         <v>88710</v>
       </c>
-      <c r="K116" s="15" t="inlineStr">
+      <c r="E119" s="345" t="n"/>
+      <c r="F119" s="345" t="n"/>
+      <c r="G119" s="345" t="n"/>
+      <c r="H119" s="345" t="n"/>
+      <c r="I119" s="345" t="n"/>
+      <c r="J119" s="345" t="n"/>
+      <c r="K119" s="345" t="n"/>
+      <c r="L119" s="345" t="n"/>
+      <c r="M119" s="345" t="n"/>
+      <c r="N119" s="15" t="n"/>
+    </row>
+    <row r="120" ht="18" customHeight="1">
+      <c r="A120" s="337" t="inlineStr">
+        <is>
+          <t>5o</t>
+        </is>
+      </c>
+      <c r="B120" s="338" t="n"/>
+      <c r="C120" s="365" t="inlineStr">
         <is>
           <t>OFICINA</t>
         </is>
       </c>
-      <c r="L116" s="15" t="n">
+      <c r="D120" s="340" t="n">
         <v>28000</v>
       </c>
-      <c r="M116" s="15" t="n"/>
-      <c r="N116" s="15" t="n"/>
-    </row>
-    <row r="117" ht="18" customHeight="1">
-      <c r="A117" s="14" t="inlineStr">
-        <is>
-          <t>2o lugar</t>
-        </is>
-      </c>
-      <c r="B117" s="15" t="n"/>
-      <c r="C117" s="15" t="n"/>
-      <c r="D117" s="15" t="n"/>
-      <c r="E117" s="15" t="n"/>
-      <c r="F117" s="15" t="n"/>
-      <c r="G117" s="15" t="n"/>
-      <c r="H117" s="15" t="n"/>
-      <c r="I117" s="15" t="n"/>
-      <c r="J117" s="15" t="n"/>
-      <c r="K117" s="15" t="n"/>
-      <c r="L117" s="15" t="n"/>
-      <c r="M117" s="15" t="n"/>
-      <c r="N117" s="15" t="n"/>
-    </row>
-    <row r="118" ht="18" customHeight="1">
-      <c r="A118" s="14" t="inlineStr">
-        <is>
-          <t>3er lugar</t>
-        </is>
-      </c>
-      <c r="B118" s="15" t="n"/>
-      <c r="C118" s="15" t="n"/>
-      <c r="D118" s="15" t="n"/>
-      <c r="E118" s="15" t="n"/>
-      <c r="F118" s="15" t="n"/>
-      <c r="G118" s="15" t="n"/>
-      <c r="H118" s="15" t="n"/>
-      <c r="I118" s="15" t="n"/>
-      <c r="J118" s="15" t="n"/>
-      <c r="K118" s="15" t="n"/>
-      <c r="L118" s="15" t="n"/>
-      <c r="M118" s="15" t="n"/>
-      <c r="N118" s="15" t="n"/>
-    </row>
-    <row r="119" ht="18" customHeight="1">
-      <c r="A119" s="14" t="inlineStr">
-        <is>
-          <t>4o lugar</t>
-        </is>
-      </c>
-      <c r="B119" s="15" t="n"/>
-      <c r="C119" s="15" t="n"/>
-      <c r="D119" s="15" t="n"/>
-      <c r="E119" s="15" t="n"/>
-      <c r="F119" s="15" t="n"/>
-      <c r="G119" s="15" t="n"/>
-      <c r="H119" s="15" t="n"/>
-      <c r="I119" s="15" t="n"/>
-      <c r="J119" s="15" t="n"/>
-      <c r="K119" s="15" t="n"/>
-      <c r="L119" s="15" t="n"/>
-      <c r="M119" s="15" t="n"/>
-      <c r="N119" s="15" t="n"/>
-    </row>
-    <row r="120" ht="18" customHeight="1">
-      <c r="A120" s="14" t="inlineStr">
-        <is>
-          <t>5o lugar</t>
-        </is>
-      </c>
-      <c r="B120" s="15" t="n"/>
-      <c r="C120" s="15" t="n"/>
-      <c r="D120" s="15" t="n"/>
-      <c r="E120" s="15" t="n"/>
-      <c r="F120" s="15" t="n"/>
-      <c r="G120" s="15" t="n"/>
-      <c r="H120" s="15" t="n"/>
-      <c r="I120" s="15" t="n"/>
-      <c r="J120" s="15" t="n"/>
-      <c r="K120" s="15" t="n"/>
-      <c r="L120" s="15" t="n"/>
-      <c r="M120" s="15" t="n"/>
+      <c r="E120" s="26" t="n"/>
+      <c r="F120" s="26" t="n"/>
+      <c r="G120" s="26" t="n"/>
+      <c r="H120" s="26" t="n"/>
+      <c r="I120" s="26" t="n"/>
+      <c r="J120" s="26" t="n"/>
+      <c r="K120" s="26" t="n"/>
+      <c r="L120" s="26" t="n"/>
+      <c r="M120" s="26" t="n"/>
       <c r="N120" s="15" t="n"/>
     </row>
     <row r="121" ht="6" customHeight="1"/>
     <row r="122">
-      <c r="A122" s="35" t="inlineStr">
+      <c r="A122" s="367" t="inlineStr">
         <is>
           <t>COBRANZA RECUPERADA</t>
         </is>
       </c>
-      <c r="B122" s="28" t="n"/>
-      <c r="C122" s="28" t="n"/>
-      <c r="D122" s="28" t="n"/>
-      <c r="E122" s="28" t="n"/>
-      <c r="F122" s="28" t="n"/>
-      <c r="G122" s="28" t="n"/>
-      <c r="H122" s="28" t="n"/>
-      <c r="I122" s="28" t="n"/>
-      <c r="J122" s="28" t="n"/>
-      <c r="K122" s="28" t="n"/>
-      <c r="L122" s="28" t="n"/>
-      <c r="M122" s="28" t="n"/>
+      <c r="B122" s="368" t="n"/>
+      <c r="C122" s="368" t="n"/>
+      <c r="D122" s="368" t="n"/>
+      <c r="E122" s="368" t="n"/>
+      <c r="F122" s="368" t="n"/>
+      <c r="G122" s="368" t="n"/>
+      <c r="H122" s="368" t="n"/>
+      <c r="I122" s="368" t="n"/>
+      <c r="J122" s="368" t="n"/>
+      <c r="K122" s="368" t="n"/>
+      <c r="L122" s="368" t="n"/>
+      <c r="M122" s="368" t="n"/>
       <c r="N122" s="28" t="n"/>
     </row>
     <row r="123" ht="20" customHeight="1">
-      <c r="A123" s="8" t="inlineStr">
+      <c r="A123" s="332" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B123" s="11" t="n">
+      <c r="B123" s="369" t="n">
         <v>94027</v>
       </c>
+      <c r="C123" s="334" t="n"/>
+      <c r="D123" s="334" t="n"/>
+      <c r="E123" s="334" t="n"/>
+      <c r="F123" s="334" t="n"/>
+      <c r="G123" s="334" t="n"/>
+      <c r="H123" s="334" t="n"/>
+      <c r="I123" s="334" t="n"/>
+      <c r="J123" s="334" t="n"/>
+      <c r="K123" s="334" t="n"/>
+      <c r="L123" s="334" t="n"/>
+      <c r="M123" s="334" t="n"/>
     </row>
     <row r="124" ht="18" customHeight="1">
-      <c r="A124" s="12" t="inlineStr">
+      <c r="A124" s="335" t="inlineStr">
         <is>
           <t>Top 5</t>
         </is>
       </c>
-      <c r="C124" s="13" t="n"/>
-      <c r="D124" s="13" t="n"/>
-      <c r="E124" s="13" t="n"/>
-      <c r="F124" s="13" t="n"/>
-      <c r="G124" s="13" t="n"/>
-      <c r="H124" s="13" t="n"/>
-      <c r="I124" s="13" t="n"/>
-      <c r="J124" s="13" t="n"/>
-      <c r="K124" s="13" t="n"/>
-      <c r="L124" s="13" t="n"/>
-      <c r="M124" s="13" t="n"/>
+      <c r="C124" s="336" t="n"/>
+      <c r="D124" s="336" t="n"/>
+      <c r="E124" s="336" t="n"/>
+      <c r="F124" s="336" t="n"/>
+      <c r="G124" s="336" t="n"/>
+      <c r="H124" s="336" t="n"/>
+      <c r="I124" s="336" t="n"/>
+      <c r="J124" s="336" t="n"/>
+      <c r="K124" s="336" t="n"/>
+      <c r="L124" s="336" t="n"/>
+      <c r="M124" s="336" t="n"/>
       <c r="N124" s="13" t="n"/>
     </row>
     <row r="125" ht="18" customHeight="1">
-      <c r="A125" s="14" t="inlineStr">
-        <is>
-          <t>1er lugar</t>
-        </is>
-      </c>
-      <c r="B125" s="15" t="n"/>
-      <c r="C125" s="15" t="n"/>
-      <c r="D125" s="15" t="n"/>
-      <c r="E125" s="15" t="n"/>
-      <c r="F125" s="15" t="n"/>
-      <c r="G125" s="15" t="n"/>
-      <c r="H125" s="15" t="n"/>
-      <c r="I125" s="15" t="n"/>
-      <c r="J125" s="15" t="n"/>
-      <c r="K125" s="15" t="n"/>
-      <c r="L125" s="15" t="n"/>
-      <c r="M125" s="15" t="n"/>
+      <c r="A125" s="337" t="inlineStr">
+        <is>
+          <t>1er</t>
+        </is>
+      </c>
+      <c r="B125" s="338" t="n"/>
+      <c r="C125" s="370" t="n"/>
+      <c r="D125" s="340" t="n"/>
+      <c r="E125" s="26" t="n"/>
+      <c r="F125" s="26" t="n"/>
+      <c r="G125" s="26" t="n"/>
+      <c r="H125" s="26" t="n"/>
+      <c r="I125" s="26" t="n"/>
+      <c r="J125" s="26" t="n"/>
+      <c r="K125" s="26" t="n"/>
+      <c r="L125" s="26" t="n"/>
+      <c r="M125" s="26" t="n"/>
       <c r="N125" s="15" t="n"/>
     </row>
     <row r="126" ht="18" customHeight="1">
-      <c r="A126" s="14" t="inlineStr">
-        <is>
-          <t>2o lugar</t>
-        </is>
-      </c>
-      <c r="B126" s="15" t="n"/>
-      <c r="C126" s="15" t="n"/>
-      <c r="D126" s="15" t="n"/>
-      <c r="E126" s="15" t="n"/>
-      <c r="F126" s="15" t="n"/>
-      <c r="G126" s="15" t="n"/>
-      <c r="H126" s="15" t="n"/>
-      <c r="I126" s="15" t="n"/>
-      <c r="J126" s="15" t="n"/>
-      <c r="K126" s="15" t="n"/>
-      <c r="L126" s="15" t="n"/>
-      <c r="M126" s="15" t="n"/>
+      <c r="A126" s="341" t="inlineStr">
+        <is>
+          <t>2o</t>
+        </is>
+      </c>
+      <c r="B126" s="342" t="n"/>
+      <c r="C126" s="371" t="n"/>
+      <c r="D126" s="344" t="n"/>
+      <c r="E126" s="345" t="n"/>
+      <c r="F126" s="345" t="n"/>
+      <c r="G126" s="345" t="n"/>
+      <c r="H126" s="345" t="n"/>
+      <c r="I126" s="345" t="n"/>
+      <c r="J126" s="345" t="n"/>
+      <c r="K126" s="345" t="n"/>
+      <c r="L126" s="345" t="n"/>
+      <c r="M126" s="345" t="n"/>
       <c r="N126" s="15" t="n"/>
     </row>
     <row r="127" ht="18" customHeight="1">
-      <c r="A127" s="14" t="inlineStr">
-        <is>
-          <t>3er lugar</t>
-        </is>
-      </c>
-      <c r="B127" s="15" t="n"/>
-      <c r="C127" s="15" t="n"/>
-      <c r="D127" s="15" t="n"/>
-      <c r="E127" s="15" t="n"/>
-      <c r="F127" s="15" t="n"/>
-      <c r="G127" s="15" t="n"/>
-      <c r="H127" s="15" t="n"/>
-      <c r="I127" s="15" t="n"/>
-      <c r="J127" s="15" t="n"/>
-      <c r="K127" s="15" t="n"/>
-      <c r="L127" s="15" t="n"/>
-      <c r="M127" s="15" t="n"/>
+      <c r="A127" s="337" t="inlineStr">
+        <is>
+          <t>3er</t>
+        </is>
+      </c>
+      <c r="B127" s="338" t="n"/>
+      <c r="C127" s="370" t="n"/>
+      <c r="D127" s="340" t="n"/>
+      <c r="E127" s="26" t="n"/>
+      <c r="F127" s="26" t="n"/>
+      <c r="G127" s="26" t="n"/>
+      <c r="H127" s="26" t="n"/>
+      <c r="I127" s="26" t="n"/>
+      <c r="J127" s="26" t="n"/>
+      <c r="K127" s="26" t="n"/>
+      <c r="L127" s="26" t="n"/>
+      <c r="M127" s="26" t="n"/>
       <c r="N127" s="15" t="n"/>
     </row>
     <row r="128" ht="18" customHeight="1">
-      <c r="A128" s="14" t="inlineStr">
-        <is>
-          <t>4o lugar</t>
-        </is>
-      </c>
-      <c r="B128" s="15" t="n"/>
-      <c r="C128" s="15" t="n"/>
-      <c r="D128" s="15" t="n"/>
-      <c r="E128" s="15" t="n"/>
-      <c r="F128" s="15" t="n"/>
-      <c r="G128" s="15" t="n"/>
-      <c r="H128" s="15" t="n"/>
-      <c r="I128" s="15" t="n"/>
-      <c r="J128" s="15" t="n"/>
-      <c r="K128" s="15" t="n"/>
-      <c r="L128" s="15" t="n"/>
-      <c r="M128" s="15" t="n"/>
+      <c r="A128" s="341" t="inlineStr">
+        <is>
+          <t>4o</t>
+        </is>
+      </c>
+      <c r="B128" s="342" t="n"/>
+      <c r="C128" s="371" t="n"/>
+      <c r="D128" s="344" t="n"/>
+      <c r="E128" s="345" t="n"/>
+      <c r="F128" s="345" t="n"/>
+      <c r="G128" s="345" t="n"/>
+      <c r="H128" s="345" t="n"/>
+      <c r="I128" s="345" t="n"/>
+      <c r="J128" s="345" t="n"/>
+      <c r="K128" s="345" t="n"/>
+      <c r="L128" s="345" t="n"/>
+      <c r="M128" s="345" t="n"/>
       <c r="N128" s="15" t="n"/>
     </row>
     <row r="129" ht="18" customHeight="1">
-      <c r="A129" s="14" t="inlineStr">
-        <is>
-          <t>5o lugar</t>
-        </is>
-      </c>
-      <c r="B129" s="15" t="n"/>
-      <c r="C129" s="15" t="n"/>
-      <c r="D129" s="15" t="n"/>
-      <c r="E129" s="15" t="n"/>
-      <c r="F129" s="15" t="n"/>
-      <c r="G129" s="15" t="n"/>
-      <c r="H129" s="15" t="n"/>
-      <c r="I129" s="15" t="n"/>
-      <c r="J129" s="15" t="n"/>
-      <c r="K129" s="15" t="n"/>
-      <c r="L129" s="15" t="n"/>
-      <c r="M129" s="15" t="n"/>
+      <c r="A129" s="337" t="inlineStr">
+        <is>
+          <t>5o</t>
+        </is>
+      </c>
+      <c r="B129" s="338" t="n"/>
+      <c r="C129" s="370" t="n"/>
+      <c r="D129" s="340" t="n"/>
+      <c r="E129" s="26" t="n"/>
+      <c r="F129" s="26" t="n"/>
+      <c r="G129" s="26" t="n"/>
+      <c r="H129" s="26" t="n"/>
+      <c r="I129" s="26" t="n"/>
+      <c r="J129" s="26" t="n"/>
+      <c r="K129" s="26" t="n"/>
+      <c r="L129" s="26" t="n"/>
+      <c r="M129" s="26" t="n"/>
       <c r="N129" s="15" t="n"/>
     </row>
     <row r="130" ht="6" customHeight="1"/>
     <row r="131">
-      <c r="A131" s="35" t="inlineStr">
+      <c r="A131" s="372" t="inlineStr">
         <is>
           <t>COBRANZA TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B131" s="28" t="n"/>
-      <c r="C131" s="28" t="n"/>
-      <c r="D131" s="28" t="n"/>
-      <c r="E131" s="28" t="n"/>
-      <c r="F131" s="28" t="n"/>
-      <c r="G131" s="28" t="n"/>
-      <c r="H131" s="28" t="n"/>
-      <c r="I131" s="28" t="n"/>
-      <c r="J131" s="28" t="n"/>
-      <c r="K131" s="28" t="n"/>
-      <c r="L131" s="28" t="n"/>
-      <c r="M131" s="28" t="n"/>
+      <c r="B131" s="373" t="n"/>
+      <c r="C131" s="373" t="n"/>
+      <c r="D131" s="373" t="n"/>
+      <c r="E131" s="373" t="n"/>
+      <c r="F131" s="373" t="n"/>
+      <c r="G131" s="373" t="n"/>
+      <c r="H131" s="373" t="n"/>
+      <c r="I131" s="373" t="n"/>
+      <c r="J131" s="373" t="n"/>
+      <c r="K131" s="373" t="n"/>
+      <c r="L131" s="373" t="n"/>
+      <c r="M131" s="373" t="n"/>
       <c r="N131" s="28" t="n"/>
     </row>
     <row r="132" ht="20" customHeight="1">
-      <c r="A132" s="16" t="inlineStr">
+      <c r="A132" s="374" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B132" s="17" t="n">
+      <c r="B132" s="375" t="n">
         <v>1251614</v>
       </c>
+      <c r="C132" s="376" t="n"/>
+      <c r="D132" s="376" t="n"/>
+      <c r="E132" s="376" t="n"/>
+      <c r="F132" s="376" t="n"/>
+      <c r="G132" s="376" t="n"/>
+      <c r="H132" s="376" t="n"/>
+      <c r="I132" s="376" t="n"/>
+      <c r="J132" s="376" t="n"/>
+      <c r="K132" s="376" t="n"/>
+      <c r="L132" s="376" t="n"/>
+      <c r="M132" s="376" t="n"/>
     </row>
     <row r="133" ht="18" customHeight="1">
-      <c r="A133" s="12" t="inlineStr">
+      <c r="A133" s="335" t="inlineStr">
         <is>
           <t>Top 5</t>
         </is>
       </c>
-      <c r="C133" s="13" t="n"/>
-      <c r="D133" s="13" t="n"/>
-      <c r="E133" s="13" t="n"/>
-      <c r="F133" s="13" t="n"/>
-      <c r="G133" s="13" t="n"/>
-      <c r="H133" s="13" t="n"/>
-      <c r="I133" s="13" t="n"/>
-      <c r="J133" s="13" t="n"/>
-      <c r="K133" s="13" t="n"/>
-      <c r="L133" s="13" t="n"/>
-      <c r="M133" s="13" t="n"/>
+      <c r="C133" s="336" t="n"/>
+      <c r="D133" s="336" t="n"/>
+      <c r="E133" s="336" t="n"/>
+      <c r="F133" s="336" t="n"/>
+      <c r="G133" s="336" t="n"/>
+      <c r="H133" s="336" t="n"/>
+      <c r="I133" s="336" t="n"/>
+      <c r="J133" s="336" t="n"/>
+      <c r="K133" s="336" t="n"/>
+      <c r="L133" s="336" t="n"/>
+      <c r="M133" s="336" t="n"/>
       <c r="N133" s="13" t="n"/>
     </row>
     <row r="134" ht="18" customHeight="1">
-      <c r="A134" s="14" t="inlineStr">
-        <is>
-          <t>1er lugar</t>
-        </is>
-      </c>
-      <c r="B134" s="15" t="n"/>
-      <c r="C134" s="15" t="inlineStr">
+      <c r="A134" s="337" t="inlineStr">
+        <is>
+          <t>1er</t>
+        </is>
+      </c>
+      <c r="B134" s="338" t="n"/>
+      <c r="C134" s="377" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
       </c>
-      <c r="D134" s="15" t="n">
+      <c r="D134" s="340" t="n">
         <v>227673</v>
       </c>
-      <c r="E134" s="15" t="inlineStr">
+      <c r="E134" s="26" t="n"/>
+      <c r="F134" s="26" t="n"/>
+      <c r="G134" s="26" t="n"/>
+      <c r="H134" s="26" t="n"/>
+      <c r="I134" s="26" t="n"/>
+      <c r="J134" s="26" t="n"/>
+      <c r="K134" s="26" t="n"/>
+      <c r="L134" s="26" t="n"/>
+      <c r="M134" s="26" t="n"/>
+      <c r="N134" s="15" t="n"/>
+    </row>
+    <row r="135" ht="18" customHeight="1">
+      <c r="A135" s="341" t="inlineStr">
+        <is>
+          <t>2o</t>
+        </is>
+      </c>
+      <c r="B135" s="342" t="n"/>
+      <c r="C135" s="378" t="inlineStr">
         <is>
           <t>JORGE</t>
         </is>
       </c>
-      <c r="F134" s="15" t="n">
+      <c r="D135" s="344" t="n">
         <v>170311</v>
       </c>
-      <c r="G134" s="15" t="inlineStr">
+      <c r="E135" s="345" t="n"/>
+      <c r="F135" s="345" t="n"/>
+      <c r="G135" s="345" t="n"/>
+      <c r="H135" s="345" t="n"/>
+      <c r="I135" s="345" t="n"/>
+      <c r="J135" s="345" t="n"/>
+      <c r="K135" s="345" t="n"/>
+      <c r="L135" s="345" t="n"/>
+      <c r="M135" s="345" t="n"/>
+      <c r="N135" s="15" t="n"/>
+    </row>
+    <row r="136" ht="18" customHeight="1">
+      <c r="A136" s="337" t="inlineStr">
+        <is>
+          <t>3er</t>
+        </is>
+      </c>
+      <c r="B136" s="338" t="n"/>
+      <c r="C136" s="377" t="inlineStr">
         <is>
           <t>V6</t>
         </is>
       </c>
-      <c r="H134" s="15" t="n">
+      <c r="D136" s="340" t="n">
         <v>153967</v>
       </c>
-      <c r="I134" s="15" t="inlineStr">
+      <c r="E136" s="26" t="n"/>
+      <c r="F136" s="26" t="n"/>
+      <c r="G136" s="26" t="n"/>
+      <c r="H136" s="26" t="n"/>
+      <c r="I136" s="26" t="n"/>
+      <c r="J136" s="26" t="n"/>
+      <c r="K136" s="26" t="n"/>
+      <c r="L136" s="26" t="n"/>
+      <c r="M136" s="26" t="n"/>
+      <c r="N136" s="15" t="n"/>
+    </row>
+    <row r="137" ht="18" customHeight="1">
+      <c r="A137" s="341" t="inlineStr">
+        <is>
+          <t>4o</t>
+        </is>
+      </c>
+      <c r="B137" s="342" t="n"/>
+      <c r="C137" s="378" t="inlineStr">
         <is>
           <t>DEPOSITO</t>
         </is>
       </c>
-      <c r="J134" s="15" t="n">
+      <c r="D137" s="344" t="n">
         <v>98765</v>
       </c>
-      <c r="K134" s="15" t="inlineStr">
+      <c r="E137" s="345" t="n"/>
+      <c r="F137" s="345" t="n"/>
+      <c r="G137" s="345" t="n"/>
+      <c r="H137" s="345" t="n"/>
+      <c r="I137" s="345" t="n"/>
+      <c r="J137" s="345" t="n"/>
+      <c r="K137" s="345" t="n"/>
+      <c r="L137" s="345" t="n"/>
+      <c r="M137" s="345" t="n"/>
+      <c r="N137" s="15" t="n"/>
+    </row>
+    <row r="138" ht="18" customHeight="1">
+      <c r="A138" s="337" t="inlineStr">
+        <is>
+          <t>5o</t>
+        </is>
+      </c>
+      <c r="B138" s="338" t="n"/>
+      <c r="C138" s="377" t="inlineStr">
         <is>
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="L134" s="15" t="n">
+      <c r="D138" s="340" t="n">
         <v>87654</v>
       </c>
-      <c r="M134" s="15" t="n"/>
-      <c r="N134" s="15" t="n"/>
-    </row>
-    <row r="135" ht="18" customHeight="1">
-      <c r="A135" s="14" t="inlineStr">
-        <is>
-          <t>2o lugar</t>
-        </is>
-      </c>
-      <c r="B135" s="15" t="n"/>
-      <c r="C135" s="15" t="n"/>
-      <c r="D135" s="15" t="n"/>
-      <c r="E135" s="15" t="n"/>
-      <c r="F135" s="15" t="n"/>
-      <c r="G135" s="15" t="n"/>
-      <c r="H135" s="15" t="n"/>
-      <c r="I135" s="15" t="n"/>
-      <c r="J135" s="15" t="n"/>
-      <c r="K135" s="15" t="n"/>
-      <c r="L135" s="15" t="n"/>
-      <c r="M135" s="15" t="n"/>
-      <c r="N135" s="15" t="n"/>
-    </row>
-    <row r="136" ht="18" customHeight="1">
-      <c r="A136" s="14" t="inlineStr">
-        <is>
-          <t>3er lugar</t>
-        </is>
-      </c>
-      <c r="B136" s="15" t="n"/>
-      <c r="C136" s="15" t="n"/>
-      <c r="D136" s="15" t="n"/>
-      <c r="E136" s="15" t="n"/>
-      <c r="F136" s="15" t="n"/>
-      <c r="G136" s="15" t="n"/>
-      <c r="H136" s="15" t="n"/>
-      <c r="I136" s="15" t="n"/>
-      <c r="J136" s="15" t="n"/>
-      <c r="K136" s="15" t="n"/>
-      <c r="L136" s="15" t="n"/>
-      <c r="M136" s="15" t="n"/>
-      <c r="N136" s="15" t="n"/>
-    </row>
-    <row r="137" ht="18" customHeight="1">
-      <c r="A137" s="14" t="inlineStr">
-        <is>
-          <t>4o lugar</t>
-        </is>
-      </c>
-      <c r="B137" s="15" t="n"/>
-      <c r="C137" s="15" t="n"/>
-      <c r="D137" s="15" t="n"/>
-      <c r="E137" s="15" t="n"/>
-      <c r="F137" s="15" t="n"/>
-      <c r="G137" s="15" t="n"/>
-      <c r="H137" s="15" t="n"/>
-      <c r="I137" s="15" t="n"/>
-      <c r="J137" s="15" t="n"/>
-      <c r="K137" s="15" t="n"/>
-      <c r="L137" s="15" t="n"/>
-      <c r="M137" s="15" t="n"/>
-      <c r="N137" s="15" t="n"/>
-    </row>
-    <row r="138" ht="18" customHeight="1">
-      <c r="A138" s="14" t="inlineStr">
-        <is>
-          <t>5o lugar</t>
-        </is>
-      </c>
-      <c r="B138" s="15" t="n"/>
-      <c r="C138" s="15" t="n"/>
-      <c r="D138" s="15" t="n"/>
-      <c r="E138" s="15" t="n"/>
-      <c r="F138" s="15" t="n"/>
-      <c r="G138" s="15" t="n"/>
-      <c r="H138" s="15" t="n"/>
-      <c r="I138" s="15" t="n"/>
-      <c r="J138" s="15" t="n"/>
-      <c r="K138" s="15" t="n"/>
-      <c r="L138" s="15" t="n"/>
-      <c r="M138" s="15" t="n"/>
+      <c r="E138" s="26" t="n"/>
+      <c r="F138" s="26" t="n"/>
+      <c r="G138" s="26" t="n"/>
+      <c r="H138" s="26" t="n"/>
+      <c r="I138" s="26" t="n"/>
+      <c r="J138" s="26" t="n"/>
+      <c r="K138" s="26" t="n"/>
+      <c r="L138" s="26" t="n"/>
+      <c r="M138" s="26" t="n"/>
       <c r="N138" s="15" t="n"/>
     </row>
     <row r="139" ht="6" customHeight="1"/>
     <row r="140">
-      <c r="A140" s="35" t="inlineStr">
+      <c r="A140" s="379" t="inlineStr">
         <is>
           <t>COBRANZA ADELANTADA F.</t>
         </is>
       </c>
-      <c r="B140" s="28" t="n"/>
-      <c r="C140" s="28" t="n"/>
-      <c r="D140" s="28" t="n"/>
-      <c r="E140" s="28" t="n"/>
-      <c r="F140" s="28" t="n"/>
-      <c r="G140" s="28" t="n"/>
-      <c r="H140" s="28" t="n"/>
-      <c r="I140" s="28" t="n"/>
-      <c r="J140" s="28" t="n"/>
-      <c r="K140" s="28" t="n"/>
-      <c r="L140" s="28" t="n"/>
-      <c r="M140" s="28" t="n"/>
+      <c r="B140" s="380" t="n"/>
+      <c r="C140" s="380" t="n"/>
+      <c r="D140" s="380" t="n"/>
+      <c r="E140" s="380" t="n"/>
+      <c r="F140" s="380" t="n"/>
+      <c r="G140" s="380" t="n"/>
+      <c r="H140" s="380" t="n"/>
+      <c r="I140" s="380" t="n"/>
+      <c r="J140" s="380" t="n"/>
+      <c r="K140" s="380" t="n"/>
+      <c r="L140" s="380" t="n"/>
+      <c r="M140" s="380" t="n"/>
       <c r="N140" s="28" t="n"/>
     </row>
     <row r="141" ht="20" customHeight="1">
-      <c r="A141" s="8" t="inlineStr">
+      <c r="A141" s="381" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B141" s="11" t="n">
+      <c r="B141" s="382" t="n">
         <v>8618</v>
       </c>
+      <c r="C141" s="383" t="n"/>
+      <c r="D141" s="383" t="n"/>
+      <c r="E141" s="383" t="n"/>
+      <c r="F141" s="383" t="n"/>
+      <c r="G141" s="383" t="n"/>
+      <c r="H141" s="383" t="n"/>
+      <c r="I141" s="383" t="n"/>
+      <c r="J141" s="383" t="n"/>
+      <c r="K141" s="383" t="n"/>
+      <c r="L141" s="383" t="n"/>
+      <c r="M141" s="383" t="n"/>
     </row>
     <row r="142" ht="18" customHeight="1">
-      <c r="A142" s="12" t="inlineStr">
+      <c r="A142" s="335" t="inlineStr">
         <is>
           <t>Top 5</t>
         </is>
       </c>
-      <c r="C142" s="13" t="n"/>
-      <c r="D142" s="13" t="n"/>
-      <c r="E142" s="13" t="n"/>
-      <c r="F142" s="13" t="n"/>
-      <c r="G142" s="13" t="n"/>
-      <c r="H142" s="13" t="n"/>
-      <c r="I142" s="13" t="n"/>
-      <c r="J142" s="13" t="n"/>
-      <c r="K142" s="13" t="n"/>
-      <c r="L142" s="13" t="n"/>
-      <c r="M142" s="13" t="n"/>
+      <c r="C142" s="336" t="n"/>
+      <c r="D142" s="336" t="n"/>
+      <c r="E142" s="336" t="n"/>
+      <c r="F142" s="336" t="n"/>
+      <c r="G142" s="336" t="n"/>
+      <c r="H142" s="336" t="n"/>
+      <c r="I142" s="336" t="n"/>
+      <c r="J142" s="336" t="n"/>
+      <c r="K142" s="336" t="n"/>
+      <c r="L142" s="336" t="n"/>
+      <c r="M142" s="336" t="n"/>
       <c r="N142" s="13" t="n"/>
     </row>
     <row r="143" ht="18" customHeight="1">
-      <c r="A143" s="14" t="inlineStr">
-        <is>
-          <t>1er lugar</t>
-        </is>
-      </c>
-      <c r="B143" s="15" t="n"/>
-      <c r="C143" s="15" t="n"/>
-      <c r="D143" s="15" t="n"/>
-      <c r="E143" s="15" t="n"/>
-      <c r="F143" s="15" t="n"/>
-      <c r="G143" s="15" t="n"/>
-      <c r="H143" s="15" t="n"/>
-      <c r="I143" s="15" t="n"/>
-      <c r="J143" s="15" t="n"/>
-      <c r="K143" s="15" t="n"/>
-      <c r="L143" s="15" t="n"/>
-      <c r="M143" s="15" t="n"/>
+      <c r="A143" s="337" t="inlineStr">
+        <is>
+          <t>1er</t>
+        </is>
+      </c>
+      <c r="B143" s="338" t="n"/>
+      <c r="C143" s="384" t="n"/>
+      <c r="D143" s="340" t="n"/>
+      <c r="E143" s="26" t="n"/>
+      <c r="F143" s="26" t="n"/>
+      <c r="G143" s="26" t="n"/>
+      <c r="H143" s="26" t="n"/>
+      <c r="I143" s="26" t="n"/>
+      <c r="J143" s="26" t="n"/>
+      <c r="K143" s="26" t="n"/>
+      <c r="L143" s="26" t="n"/>
+      <c r="M143" s="26" t="n"/>
       <c r="N143" s="15" t="n"/>
     </row>
     <row r="144" ht="18" customHeight="1">
-      <c r="A144" s="14" t="inlineStr">
-        <is>
-          <t>2o lugar</t>
-        </is>
-      </c>
-      <c r="B144" s="15" t="n"/>
-      <c r="C144" s="15" t="n"/>
-      <c r="D144" s="15" t="n"/>
-      <c r="E144" s="15" t="n"/>
-      <c r="F144" s="15" t="n"/>
-      <c r="G144" s="15" t="n"/>
-      <c r="H144" s="15" t="n"/>
-      <c r="I144" s="15" t="n"/>
-      <c r="J144" s="15" t="n"/>
-      <c r="K144" s="15" t="n"/>
-      <c r="L144" s="15" t="n"/>
-      <c r="M144" s="15" t="n"/>
+      <c r="A144" s="341" t="inlineStr">
+        <is>
+          <t>2o</t>
+        </is>
+      </c>
+      <c r="B144" s="342" t="n"/>
+      <c r="C144" s="385" t="n"/>
+      <c r="D144" s="344" t="n"/>
+      <c r="E144" s="345" t="n"/>
+      <c r="F144" s="345" t="n"/>
+      <c r="G144" s="345" t="n"/>
+      <c r="H144" s="345" t="n"/>
+      <c r="I144" s="345" t="n"/>
+      <c r="J144" s="345" t="n"/>
+      <c r="K144" s="345" t="n"/>
+      <c r="L144" s="345" t="n"/>
+      <c r="M144" s="345" t="n"/>
       <c r="N144" s="15" t="n"/>
     </row>
     <row r="145" ht="18" customHeight="1">
-      <c r="A145" s="14" t="inlineStr">
-        <is>
-          <t>3er lugar</t>
-        </is>
-      </c>
-      <c r="B145" s="15" t="n"/>
-      <c r="C145" s="15" t="n"/>
-      <c r="D145" s="15" t="n"/>
-      <c r="E145" s="15" t="n"/>
-      <c r="F145" s="15" t="n"/>
-      <c r="G145" s="15" t="n"/>
-      <c r="H145" s="15" t="n"/>
-      <c r="I145" s="15" t="n"/>
-      <c r="J145" s="15" t="n"/>
-      <c r="K145" s="15" t="n"/>
-      <c r="L145" s="15" t="n"/>
-      <c r="M145" s="15" t="n"/>
+      <c r="A145" s="337" t="inlineStr">
+        <is>
+          <t>3er</t>
+        </is>
+      </c>
+      <c r="B145" s="338" t="n"/>
+      <c r="C145" s="384" t="n"/>
+      <c r="D145" s="340" t="n"/>
+      <c r="E145" s="26" t="n"/>
+      <c r="F145" s="26" t="n"/>
+      <c r="G145" s="26" t="n"/>
+      <c r="H145" s="26" t="n"/>
+      <c r="I145" s="26" t="n"/>
+      <c r="J145" s="26" t="n"/>
+      <c r="K145" s="26" t="n"/>
+      <c r="L145" s="26" t="n"/>
+      <c r="M145" s="26" t="n"/>
       <c r="N145" s="15" t="n"/>
     </row>
     <row r="146" ht="18" customHeight="1">
-      <c r="A146" s="14" t="inlineStr">
-        <is>
-          <t>4o lugar</t>
-        </is>
-      </c>
-      <c r="B146" s="15" t="n"/>
-      <c r="C146" s="15" t="n"/>
-      <c r="D146" s="15" t="n"/>
-      <c r="E146" s="15" t="n"/>
-      <c r="F146" s="15" t="n"/>
-      <c r="G146" s="15" t="n"/>
-      <c r="H146" s="15" t="n"/>
-      <c r="I146" s="15" t="n"/>
-      <c r="J146" s="15" t="n"/>
-      <c r="K146" s="15" t="n"/>
-      <c r="L146" s="15" t="n"/>
-      <c r="M146" s="15" t="n"/>
+      <c r="A146" s="341" t="inlineStr">
+        <is>
+          <t>4o</t>
+        </is>
+      </c>
+      <c r="B146" s="342" t="n"/>
+      <c r="C146" s="385" t="n"/>
+      <c r="D146" s="344" t="n"/>
+      <c r="E146" s="345" t="n"/>
+      <c r="F146" s="345" t="n"/>
+      <c r="G146" s="345" t="n"/>
+      <c r="H146" s="345" t="n"/>
+      <c r="I146" s="345" t="n"/>
+      <c r="J146" s="345" t="n"/>
+      <c r="K146" s="345" t="n"/>
+      <c r="L146" s="345" t="n"/>
+      <c r="M146" s="345" t="n"/>
       <c r="N146" s="15" t="n"/>
     </row>
     <row r="147" ht="18" customHeight="1">
-      <c r="A147" s="14" t="inlineStr">
-        <is>
-          <t>5o lugar</t>
-        </is>
-      </c>
-      <c r="B147" s="15" t="n"/>
-      <c r="C147" s="15" t="n"/>
-      <c r="D147" s="15" t="n"/>
-      <c r="E147" s="15" t="n"/>
-      <c r="F147" s="15" t="n"/>
-      <c r="G147" s="15" t="n"/>
-      <c r="H147" s="15" t="n"/>
-      <c r="I147" s="15" t="n"/>
-      <c r="J147" s="15" t="n"/>
-      <c r="K147" s="15" t="n"/>
-      <c r="L147" s="15" t="n"/>
-      <c r="M147" s="15" t="n"/>
+      <c r="A147" s="337" t="inlineStr">
+        <is>
+          <t>5o</t>
+        </is>
+      </c>
+      <c r="B147" s="338" t="n"/>
+      <c r="C147" s="384" t="n"/>
+      <c r="D147" s="340" t="n"/>
+      <c r="E147" s="26" t="n"/>
+      <c r="F147" s="26" t="n"/>
+      <c r="G147" s="26" t="n"/>
+      <c r="H147" s="26" t="n"/>
+      <c r="I147" s="26" t="n"/>
+      <c r="J147" s="26" t="n"/>
+      <c r="K147" s="26" t="n"/>
+      <c r="L147" s="26" t="n"/>
+      <c r="M147" s="26" t="n"/>
       <c r="N147" s="15" t="n"/>
     </row>
     <row r="148" ht="6" customHeight="1"/>
     <row r="149">
-      <c r="A149" s="82" t="inlineStr">
+      <c r="A149" s="386" t="inlineStr">
         <is>
           <t>PROYECCIÓN FEBRERO → FEBRERO</t>
         </is>
       </c>
-      <c r="B149" s="28" t="n"/>
-      <c r="C149" s="28" t="n"/>
-      <c r="D149" s="28" t="n"/>
-      <c r="E149" s="28" t="n"/>
-      <c r="F149" s="28" t="n"/>
-      <c r="G149" s="28" t="n"/>
-      <c r="H149" s="28" t="n"/>
-      <c r="I149" s="28" t="n"/>
-      <c r="J149" s="28" t="n"/>
-      <c r="K149" s="28" t="n"/>
-      <c r="L149" s="28" t="n"/>
-      <c r="M149" s="28" t="n"/>
+      <c r="B149" s="387" t="n"/>
+      <c r="C149" s="387" t="n"/>
+      <c r="D149" s="387" t="n"/>
+      <c r="E149" s="387" t="n"/>
+      <c r="F149" s="387" t="n"/>
+      <c r="G149" s="387" t="n"/>
+      <c r="H149" s="387" t="n"/>
+      <c r="I149" s="387" t="n"/>
+      <c r="J149" s="387" t="n"/>
+      <c r="K149" s="387" t="n"/>
+      <c r="L149" s="387" t="n"/>
+      <c r="M149" s="387" t="n"/>
       <c r="N149" s="28" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="19" t="inlineStr">
-        <is>
-          <t>Proyección FEBRERO</t>
-        </is>
-      </c>
-      <c r="B150" s="20" t="n">
+      <c r="A150" s="332" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B150" s="333" t="n">
         <v>1158184</v>
       </c>
-    </row>
-    <row r="152" ht="14" customHeight="1"/>
+      <c r="C150" s="334" t="n"/>
+      <c r="D150" s="334" t="n"/>
+      <c r="E150" s="334" t="n"/>
+      <c r="F150" s="334" t="n"/>
+      <c r="G150" s="334" t="n"/>
+      <c r="H150" s="334" t="n"/>
+      <c r="I150" s="334" t="n"/>
+      <c r="J150" s="334" t="n"/>
+      <c r="K150" s="334" t="n"/>
+      <c r="L150" s="334" t="n"/>
+      <c r="M150" s="334" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="388" t="inlineStr">
+        <is>
+          <t>Top 5</t>
+        </is>
+      </c>
+      <c r="C151" s="389" t="n"/>
+      <c r="D151" s="389" t="n"/>
+      <c r="E151" s="389" t="n"/>
+      <c r="F151" s="389" t="n"/>
+      <c r="G151" s="389" t="n"/>
+      <c r="H151" s="389" t="n"/>
+      <c r="I151" s="389" t="n"/>
+      <c r="J151" s="389" t="n"/>
+      <c r="K151" s="389" t="n"/>
+      <c r="L151" s="389" t="n"/>
+      <c r="M151" s="389" t="n"/>
+    </row>
+    <row r="152" ht="14" customHeight="1">
+      <c r="A152" s="337" t="inlineStr">
+        <is>
+          <t>1er</t>
+        </is>
+      </c>
+      <c r="B152" s="338" t="n"/>
+      <c r="C152" s="390" t="n"/>
+      <c r="D152" s="391" t="n"/>
+      <c r="E152" s="70" t="n"/>
+      <c r="F152" s="70" t="n"/>
+      <c r="G152" s="70" t="n"/>
+      <c r="H152" s="70" t="n"/>
+      <c r="I152" s="70" t="n"/>
+      <c r="J152" s="70" t="n"/>
+      <c r="K152" s="70" t="n"/>
+      <c r="L152" s="70" t="n"/>
+      <c r="M152" s="70" t="n"/>
+    </row>
     <row r="153" ht="22" customHeight="1">
-      <c r="A153" s="4" t="inlineStr">
-        <is>
-          <t>MARZO 2026</t>
-        </is>
-      </c>
+      <c r="A153" s="341" t="inlineStr">
+        <is>
+          <t>2o</t>
+        </is>
+      </c>
+      <c r="B153" s="342" t="n"/>
+      <c r="C153" s="392" t="n"/>
+      <c r="D153" s="393" t="n"/>
+      <c r="E153" s="394" t="n"/>
+      <c r="F153" s="394" t="n"/>
+      <c r="G153" s="394" t="n"/>
+      <c r="H153" s="394" t="n"/>
+      <c r="I153" s="394" t="n"/>
+      <c r="J153" s="394" t="n"/>
+      <c r="K153" s="394" t="n"/>
+      <c r="L153" s="394" t="n"/>
+      <c r="M153" s="394" t="n"/>
     </row>
     <row r="154" ht="28" customHeight="1">
-      <c r="A154" s="5" t="inlineStr">
-        <is>
-          <t>CONCEPTO</t>
-        </is>
-      </c>
-      <c r="B154" s="5" t="inlineStr">
+      <c r="A154" s="337" t="inlineStr">
+        <is>
+          <t>3er</t>
+        </is>
+      </c>
+      <c r="B154" s="338" t="inlineStr">
         <is>
           <t>TOTAL ($)</t>
         </is>
       </c>
-      <c r="C154" s="5" t="inlineStr">
+      <c r="C154" s="339" t="inlineStr">
         <is>
           <t>TOP 1</t>
         </is>
       </c>
-      <c r="D154" s="5" t="inlineStr">
+      <c r="D154" s="395" t="inlineStr">
         <is>
           <t>TOP 2</t>
         </is>
       </c>
-      <c r="E154" s="5" t="inlineStr">
+      <c r="E154" s="396" t="inlineStr">
         <is>
           <t>TOP 3</t>
         </is>
       </c>
-      <c r="F154" s="5" t="inlineStr">
+      <c r="F154" s="396" t="inlineStr">
         <is>
           <t>TOP 4</t>
         </is>
       </c>
-      <c r="G154" s="5" t="inlineStr">
+      <c r="G154" s="396" t="inlineStr">
         <is>
           <t>TOP 5</t>
         </is>
       </c>
-      <c r="H154" s="5" t="inlineStr">
+      <c r="H154" s="396" t="inlineStr">
         <is>
           <t>% TOP 1</t>
         </is>
       </c>
-      <c r="I154" s="5" t="inlineStr">
+      <c r="I154" s="396" t="inlineStr">
         <is>
           <t>% TOP 2</t>
         </is>
       </c>
-      <c r="J154" s="5" t="inlineStr">
+      <c r="J154" s="396" t="inlineStr">
         <is>
           <t>% TOP 3</t>
         </is>
       </c>
-      <c r="K154" s="5" t="inlineStr">
+      <c r="K154" s="396" t="inlineStr">
         <is>
           <t>% TOP 4</t>
         </is>
       </c>
-      <c r="L154" s="5" t="inlineStr">
+      <c r="L154" s="396" t="inlineStr">
         <is>
           <t>% TOP 5</t>
         </is>
       </c>
-      <c r="M154" s="5" t="inlineStr">
+      <c r="M154" s="396" t="inlineStr">
         <is>
           <t>% ACUM.</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="35" t="inlineStr">
-        <is>
-          <t>DATOS GENERALES</t>
-        </is>
-      </c>
-      <c r="B155" s="28" t="n"/>
-      <c r="C155" s="28" t="n"/>
-      <c r="D155" s="28" t="n"/>
-      <c r="E155" s="28" t="n"/>
-      <c r="F155" s="28" t="n"/>
-      <c r="G155" s="28" t="n"/>
-      <c r="H155" s="28" t="n"/>
-      <c r="I155" s="28" t="n"/>
-      <c r="J155" s="28" t="n"/>
-      <c r="K155" s="28" t="n"/>
-      <c r="L155" s="28" t="n"/>
-      <c r="M155" s="28" t="n"/>
+      <c r="A155" s="397" t="inlineStr">
+        <is>
+          <t>4o</t>
+        </is>
+      </c>
+      <c r="B155" s="398" t="n"/>
+      <c r="C155" s="399" t="n"/>
+      <c r="D155" s="400" t="n"/>
+      <c r="E155" s="401" t="n"/>
+      <c r="F155" s="401" t="n"/>
+      <c r="G155" s="401" t="n"/>
+      <c r="H155" s="401" t="n"/>
+      <c r="I155" s="401" t="n"/>
+      <c r="J155" s="401" t="n"/>
+      <c r="K155" s="401" t="n"/>
+      <c r="L155" s="401" t="n"/>
+      <c r="M155" s="401" t="n"/>
       <c r="N155" s="28" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="8" t="inlineStr">
-        <is>
-          <t>Mes</t>
-        </is>
-      </c>
-      <c r="B156" s="9" t="inlineStr">
+      <c r="A156" s="337" t="inlineStr">
+        <is>
+          <t>5o</t>
+        </is>
+      </c>
+      <c r="B156" s="338" t="inlineStr">
         <is>
           <t>MARZO</t>
         </is>
       </c>
-      <c r="E156" s="8" t="inlineStr">
+      <c r="C156" s="390" t="n"/>
+      <c r="D156" s="391" t="n"/>
+      <c r="E156" s="16" t="inlineStr">
         <is>
           <t>Año</t>
         </is>
       </c>
-      <c r="F156" s="9" t="inlineStr">
+      <c r="F156" s="402" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
+      <c r="G156" s="70" t="n"/>
+      <c r="H156" s="70" t="n"/>
+      <c r="I156" s="70" t="n"/>
+      <c r="J156" s="70" t="n"/>
+      <c r="K156" s="70" t="n"/>
+      <c r="L156" s="70" t="n"/>
+      <c r="M156" s="70" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="8" t="inlineStr">
@@ -19256,7 +19910,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="258">
+  <mergeCells count="259">
     <mergeCell ref="A362:N362"/>
     <mergeCell ref="A913:N913"/>
     <mergeCell ref="B231:D231"/>
@@ -19490,6 +20144,7 @@
     <mergeCell ref="A384:B384"/>
     <mergeCell ref="A456:N456"/>
     <mergeCell ref="A714:N714"/>
+    <mergeCell ref="A151:B151"/>
     <mergeCell ref="A393:B393"/>
     <mergeCell ref="A723:N723"/>
     <mergeCell ref="A779:N779"/>

</xml_diff>